<commit_message>
FINAL BOM UPDATED WITH MASS AND CAD FINALS NEED TO FINALIZE BOM PRICE TOTAL
</commit_message>
<xml_diff>
--- a/bom/BOM_hado_titan_v3.xlsx
+++ b/bom/BOM_hado_titan_v3.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="91" uniqueCount="74">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="85" uniqueCount="71">
   <si>
     <t>BOM — Haso Titan (India sourcing: Robu.in + Zerodrag) — buffered pricing</t>
   </si>
@@ -85,13 +85,16 @@
     <t>Drivetrain (x2 sides)</t>
   </si>
   <si>
-    <t>Zerodrag — zerodrag.in/collections/drone-motors</t>
-  </si>
-  <si>
-    <t>EasyMech Heavy Duty 152mm Disc Wheel (4pc set)</t>
-  </si>
-  <si>
-    <t>https://robu.in/product/easymech-heavy-dutyhd-disc-wheel-150mm-dia-gray-1pcs/</t>
+    <t>SURPASS HOBBY 3660 ROCKET sensoreless waterproof motor</t>
+  </si>
+  <si>
+    <t>https://www.electropi.in/surpass-hobby-3660-rocket-sensoreless-waterproof-motor-3175-shaft-40-gold-plated-connectors-1750-kv</t>
+  </si>
+  <si>
+    <t>EasyMech 100mm Modified Heavy Duty Disc Wheel Gray 2 Pc Set</t>
+  </si>
+  <si>
+    <t>https://robu.in/product/modified-heavy-dutyhd-disc-wheel-100mm-dia-2pc-grey-color/</t>
   </si>
   <si>
     <t>Wheel hub coupling</t>
@@ -124,10 +127,10 @@
     <t>https://robu.in/product/flysky-fs-i6x-2-4ghz-10ch-afhds-2a-rc-transmitter-with-fs-ia10b-2-4ghz-10ch-receiver/</t>
   </si>
   <si>
-    <t>Pro-Range 22.2V 5200mAh 35C 6S LiPo battery</t>
-  </si>
-  <si>
-    <t>https://robu.in/product/orange-5200mah-6s-35c-22-2-v-lithium-polymer-battery-pack-li-po-copy/</t>
+    <t>CNHL 5200mAh 22.2V 6S 90C Racing Series Lipo Battery (EC5)</t>
+  </si>
+  <si>
+    <t>https://www.uavstore.in/cnhl-5200mah-22-2v-6s-90c-racing-series-lipo-battery-ec5/</t>
   </si>
   <si>
     <t>Main power switch</t>
@@ -196,22 +199,13 @@
     <t>Main Chasis &amp; Weapon Drum</t>
   </si>
   <si>
-    <t>CASE</t>
-  </si>
-  <si>
-    <t>150 / Kg</t>
+    <t>CASE UHMWPE</t>
   </si>
   <si>
     <t>LOCAL HARDWARE</t>
   </si>
   <si>
-    <t>WEAPON DRUM (CNC)</t>
-  </si>
-  <si>
-    <t>ARMOUR (CNC)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">GRAND TOTAL </t>
+    <t>TOTAL</t>
   </si>
   <si>
     <t>GRAND TOTAL IN USD APPROX</t>
@@ -224,9 +218,6 @@
   </si>
   <si>
     <t>Green = confirmed real product/price (Zerodrag QPT motors, Zerodrag AM32 ESC, FlySky combo).</t>
-  </si>
-  <si>
-    <t>Purple = a part whose exact size isn't decided yet — priced avg</t>
   </si>
   <si>
     <t>purpose, so the budget already has headroom built in rather than needing revision upward later.</t>
@@ -311,9 +302,27 @@
       <name val="Arial"/>
     </font>
     <font>
+      <i/>
+      <sz val="11.0"/>
+      <color rgb="FF93C47D"/>
+      <name val="Rubik"/>
+    </font>
+    <font>
+      <i/>
+      <sz val="11.0"/>
+      <color rgb="FF93C47D"/>
+      <name val="&quot;Plus Jakarta Sans&quot;"/>
+    </font>
+    <font>
       <sz val="11.0"/>
       <color rgb="FF1E8449"/>
       <name val="Arial"/>
+    </font>
+    <font>
+      <i/>
+      <sz val="11.0"/>
+      <color rgb="FF6AA84F"/>
+      <name val="Inter"/>
     </font>
     <font>
       <sz val="8.0"/>
@@ -330,22 +339,6 @@
       <color theme="1"/>
       <name val="Calibri"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11.0"/>
-      <color rgb="FFFFFFFF"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11.0"/>
-      <color rgb="FF000000"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11.0"/>
-      <color rgb="FF000000"/>
-      <name val="Arial"/>
     </font>
   </fonts>
   <fills count="8">
@@ -369,20 +362,20 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFF3F3F3"/>
-        <bgColor rgb="FFF3F3F3"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor rgb="FFFFFFFF"/>
         <bgColor rgb="FFFFFFFF"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFCE4D6"/>
-        <bgColor rgb="FFFCE4D6"/>
+        <fgColor rgb="FFB6D7A8"/>
+        <bgColor rgb="FFB6D7A8"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF38761D"/>
+        <bgColor rgb="FF38761D"/>
       </patternFill>
     </fill>
     <fill>
@@ -412,7 +405,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="36">
+  <cellXfs count="32">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -443,6 +436,9 @@
     <xf borderId="1" fillId="0" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
+    <xf borderId="1" fillId="0" fontId="7" numFmtId="3" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
+      <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
+    </xf>
     <xf borderId="1" fillId="0" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -467,52 +463,37 @@
     <xf borderId="1" fillId="3" fontId="4" numFmtId="3" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1" applyNumberFormat="1">
       <alignment shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
-    <xf borderId="1" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="0" fillId="4" fontId="12" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
+      <alignment readingOrder="0"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="13" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0"/>
+    </xf>
+    <xf borderId="1" fillId="0" fontId="14" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment shrinkToFit="0" vertical="bottom" wrapText="0"/>
+    </xf>
+    <xf borderId="0" fillId="4" fontId="15" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
+      <alignment readingOrder="0"/>
+    </xf>
+    <xf borderId="1" fillId="0" fontId="16" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment shrinkToFit="0" vertical="bottom" wrapText="0"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="17" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="18" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0"/>
+    </xf>
+    <xf borderId="1" fillId="5" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
-    </xf>
-    <xf borderId="1" fillId="0" fontId="7" numFmtId="3" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
-    </xf>
-    <xf borderId="1" fillId="0" fontId="12" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment shrinkToFit="0" vertical="bottom" wrapText="0"/>
-    </xf>
-    <xf borderId="1" fillId="0" fontId="13" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment shrinkToFit="0" vertical="bottom" wrapText="0"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="14" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="15" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0"/>
-    </xf>
-    <xf borderId="0" fillId="4" fontId="16" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
-      <alignment shrinkToFit="0" vertical="bottom" wrapText="0"/>
-    </xf>
-    <xf borderId="0" fillId="5" fontId="17" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
-    </xf>
-    <xf borderId="0" fillId="5" fontId="18" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
-    </xf>
-    <xf borderId="0" fillId="5" fontId="18" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
-      <alignment shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
     <xf borderId="1" fillId="6" fontId="7" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
-    <xf borderId="1" fillId="6" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="1" fillId="7" fontId="4" numFmtId="2" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1" applyNumberFormat="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
-    <xf borderId="1" fillId="6" fontId="4" numFmtId="3" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1" applyNumberFormat="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
-    </xf>
-    <xf borderId="1" fillId="6" fontId="4" numFmtId="3" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1" applyNumberFormat="1">
-      <alignment shrinkToFit="0" vertical="bottom" wrapText="0"/>
-    </xf>
-    <xf borderId="1" fillId="0" fontId="4" numFmtId="2" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
-      <alignment shrinkToFit="0" vertical="bottom" wrapText="0"/>
-    </xf>
-    <xf borderId="0" fillId="7" fontId="14" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
+    <xf borderId="0" fillId="7" fontId="17" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
       <alignment readingOrder="0"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
@@ -525,18 +506,7 @@
   <cellStyles count="1">
     <cellStyle xfId="0" name="Normal" builtinId="0"/>
   </cellStyles>
-  <dxfs count="1">
-    <dxf>
-      <font/>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFB7E1CD"/>
-          <bgColor rgb="FFB7E1CD"/>
-        </patternFill>
-      </fill>
-      <border/>
-    </dxf>
-  </dxfs>
+  <dxfs count="0"/>
 </styleSheet>
 </file>
 
@@ -807,323 +777,268 @@
         <v>5509.0</v>
       </c>
       <c r="E5" s="8">
-        <f t="shared" ref="E5:E10" si="1">C5*D5</f>
+        <f t="shared" ref="E5:E6" si="1">C5*D5</f>
         <v>5509</v>
       </c>
-      <c r="F5" s="9">
+      <c r="F5" s="9"/>
+      <c r="G5" s="10">
         <v>530.0</v>
       </c>
-      <c r="G5" s="8">
-        <f t="shared" ref="G5:G10" si="2">C5*F5</f>
-        <v>530</v>
-      </c>
-      <c r="H5" s="10" t="s">
+      <c r="H5" s="11" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="11"/>
-      <c r="B6" s="12" t="s">
+      <c r="A6" s="12"/>
+      <c r="B6" s="13" t="s">
         <v>12</v>
       </c>
       <c r="C6" s="6">
         <v>1.0</v>
       </c>
-      <c r="D6" s="13">
+      <c r="D6" s="14">
         <v>500.0</v>
       </c>
       <c r="E6" s="8">
         <f t="shared" si="1"/>
         <v>500</v>
       </c>
-      <c r="F6" s="6">
-        <v>45.0</v>
-      </c>
-      <c r="G6" s="8">
-        <f t="shared" si="2"/>
-        <v>45</v>
-      </c>
-      <c r="H6" s="14" t="s">
+      <c r="F6" s="6"/>
+      <c r="G6" s="8"/>
+      <c r="H6" s="15" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="11"/>
-      <c r="B7" s="12" t="s">
+      <c r="A7" s="12"/>
+      <c r="B7" s="13" t="s">
         <v>14</v>
       </c>
       <c r="C7" s="6">
         <v>1.0</v>
       </c>
-      <c r="D7" s="13">
+      <c r="D7" s="14">
         <v>700.0</v>
       </c>
-      <c r="E7" s="8">
-        <f t="shared" si="1"/>
-        <v>700</v>
-      </c>
-      <c r="F7" s="6">
-        <v>110.0</v>
-      </c>
-      <c r="G7" s="8">
-        <f t="shared" si="2"/>
-        <v>110</v>
-      </c>
-      <c r="H7" s="14" t="s">
+      <c r="E7" s="10">
+        <v>700.0</v>
+      </c>
+      <c r="F7" s="6"/>
+      <c r="G7" s="8"/>
+      <c r="H7" s="15" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="11"/>
-      <c r="B8" s="12" t="s">
+      <c r="A8" s="12"/>
+      <c r="B8" s="13" t="s">
         <v>16</v>
       </c>
       <c r="C8" s="6">
         <v>1.0</v>
       </c>
-      <c r="D8" s="13">
+      <c r="D8" s="14">
         <v>300.0</v>
       </c>
       <c r="E8" s="8">
-        <f t="shared" si="1"/>
+        <f t="shared" ref="E8:E10" si="2">C8*D8</f>
         <v>300</v>
       </c>
-      <c r="F8" s="6">
-        <v>35.0</v>
-      </c>
-      <c r="G8" s="8">
-        <f t="shared" si="2"/>
-        <v>35</v>
-      </c>
-      <c r="H8" s="14" t="s">
+      <c r="F8" s="6"/>
+      <c r="G8" s="8"/>
+      <c r="H8" s="15" t="s">
         <v>17</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="11"/>
-      <c r="B9" s="12" t="s">
+      <c r="A9" s="12"/>
+      <c r="B9" s="13" t="s">
         <v>18</v>
       </c>
       <c r="C9" s="6">
         <v>2.0</v>
       </c>
-      <c r="D9" s="13">
+      <c r="D9" s="14">
         <v>189.0</v>
       </c>
       <c r="E9" s="8">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>378</v>
       </c>
-      <c r="F9" s="6">
-        <v>20.0</v>
-      </c>
-      <c r="G9" s="8">
-        <f t="shared" si="2"/>
-        <v>40</v>
-      </c>
-      <c r="H9" s="14" t="s">
+      <c r="F9" s="6"/>
+      <c r="G9" s="8"/>
+      <c r="H9" s="15" t="s">
         <v>19</v>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="11"/>
-      <c r="B10" s="12" t="s">
+      <c r="A10" s="12"/>
+      <c r="B10" s="13" t="s">
         <v>20</v>
       </c>
       <c r="C10" s="6">
         <v>1.0</v>
       </c>
-      <c r="D10" s="13">
+      <c r="D10" s="14">
         <v>700.0</v>
       </c>
       <c r="E10" s="8">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>700</v>
       </c>
-      <c r="F10" s="6">
-        <v>180.0</v>
-      </c>
-      <c r="G10" s="8">
-        <f t="shared" si="2"/>
-        <v>180</v>
-      </c>
-      <c r="H10" s="14" t="s">
+      <c r="F10" s="6"/>
+      <c r="G10" s="8"/>
+      <c r="H10" s="15" t="s">
         <v>21</v>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="15"/>
-      <c r="B11" s="16" t="s">
+      <c r="A11" s="16"/>
+      <c r="B11" s="17" t="s">
         <v>22</v>
       </c>
-      <c r="C11" s="15"/>
-      <c r="D11" s="15"/>
-      <c r="E11" s="17">
+      <c r="C11" s="16"/>
+      <c r="D11" s="16"/>
+      <c r="E11" s="18">
         <f>SUM(E5:E10)</f>
         <v>8087</v>
       </c>
-      <c r="F11" s="15"/>
-      <c r="G11" s="17">
-        <f>SUM(G5:G10)</f>
-        <v>940</v>
-      </c>
-      <c r="H11" s="15"/>
+      <c r="F11" s="16"/>
+      <c r="G11" s="18"/>
+      <c r="H11" s="16"/>
     </row>
     <row r="12">
       <c r="A12" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="B12" s="5" t="s">
-        <v>10</v>
+      <c r="B12" s="19" t="s">
+        <v>24</v>
       </c>
       <c r="C12" s="6">
         <v>2.0</v>
       </c>
       <c r="D12" s="7">
-        <v>5509.0</v>
+        <v>2100.0</v>
       </c>
       <c r="E12" s="8">
         <f t="shared" ref="E12:E16" si="3">C12*D12</f>
-        <v>11018</v>
-      </c>
-      <c r="F12" s="9">
-        <v>530.0</v>
-      </c>
-      <c r="G12" s="8">
-        <f>C12*F12</f>
-        <v>1060</v>
-      </c>
-      <c r="H12" s="14" t="s">
-        <v>24</v>
+        <v>4200</v>
+      </c>
+      <c r="F12" s="9"/>
+      <c r="G12" s="10">
+        <v>976.0</v>
+      </c>
+      <c r="H12" s="11" t="s">
+        <v>25</v>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="11"/>
-      <c r="B13" s="18" t="s">
-        <v>25</v>
+      <c r="A13" s="12"/>
+      <c r="B13" s="20" t="s">
+        <v>26</v>
       </c>
       <c r="C13" s="6">
         <v>1.0</v>
       </c>
       <c r="D13" s="7">
-        <v>1145.0</v>
+        <v>1265.0</v>
       </c>
       <c r="E13" s="8">
         <f t="shared" si="3"/>
-        <v>1145</v>
-      </c>
-      <c r="F13" s="6">
-        <v>220.0</v>
-      </c>
-      <c r="G13" s="19">
-        <v>980.0</v>
-      </c>
-      <c r="H13" s="10" t="s">
-        <v>26</v>
+        <v>1265</v>
+      </c>
+      <c r="F13" s="9"/>
+      <c r="G13" s="10">
+        <v>432.0</v>
+      </c>
+      <c r="H13" s="11" t="s">
+        <v>27</v>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="11"/>
-      <c r="B14" s="12" t="s">
-        <v>27</v>
+      <c r="A14" s="12"/>
+      <c r="B14" s="13" t="s">
+        <v>28</v>
       </c>
       <c r="C14" s="6">
         <v>2.0</v>
       </c>
-      <c r="D14" s="13">
+      <c r="D14" s="14">
         <v>400.0</v>
       </c>
       <c r="E14" s="8">
         <f t="shared" si="3"/>
         <v>800</v>
       </c>
-      <c r="F14" s="6">
-        <v>60.0</v>
-      </c>
-      <c r="G14" s="8">
-        <f t="shared" ref="G14:G16" si="4">C14*F14</f>
-        <v>120</v>
-      </c>
-      <c r="H14" s="14" t="s">
-        <v>28</v>
+      <c r="F14" s="6"/>
+      <c r="G14" s="8"/>
+      <c r="H14" s="15" t="s">
+        <v>29</v>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="11"/>
-      <c r="B15" s="12" t="s">
-        <v>29</v>
+      <c r="A15" s="12"/>
+      <c r="B15" s="13" t="s">
+        <v>30</v>
       </c>
       <c r="C15" s="6">
         <v>4.0</v>
       </c>
-      <c r="D15" s="13">
+      <c r="D15" s="14">
         <v>189.0</v>
       </c>
       <c r="E15" s="8">
         <f t="shared" si="3"/>
         <v>756</v>
       </c>
-      <c r="F15" s="6">
-        <v>25.0</v>
-      </c>
-      <c r="G15" s="8">
-        <f t="shared" si="4"/>
-        <v>100</v>
-      </c>
-      <c r="H15" s="14" t="s">
+      <c r="F15" s="6"/>
+      <c r="G15" s="8"/>
+      <c r="H15" s="15" t="s">
         <v>19</v>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="11"/>
-      <c r="B16" s="12" t="s">
-        <v>30</v>
+      <c r="A16" s="12"/>
+      <c r="B16" s="13" t="s">
+        <v>31</v>
       </c>
       <c r="C16" s="6">
         <v>2.0</v>
       </c>
-      <c r="D16" s="13">
+      <c r="D16" s="14">
         <v>300.0</v>
       </c>
       <c r="E16" s="8">
         <f t="shared" si="3"/>
         <v>600</v>
       </c>
-      <c r="F16" s="6">
-        <v>90.0</v>
-      </c>
-      <c r="G16" s="8">
-        <f t="shared" si="4"/>
-        <v>180</v>
-      </c>
-      <c r="H16" s="14" t="s">
+      <c r="F16" s="6"/>
+      <c r="G16" s="8"/>
+      <c r="H16" s="15" t="s">
         <v>21</v>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="15"/>
-      <c r="B17" s="16" t="s">
-        <v>31</v>
-      </c>
-      <c r="C17" s="15"/>
-      <c r="D17" s="15"/>
-      <c r="E17" s="17">
+      <c r="A17" s="16"/>
+      <c r="B17" s="17" t="s">
+        <v>32</v>
+      </c>
+      <c r="C17" s="16"/>
+      <c r="D17" s="16"/>
+      <c r="E17" s="18">
         <f>SUM(E12:E16)</f>
-        <v>14319</v>
-      </c>
-      <c r="F17" s="15"/>
-      <c r="G17" s="17">
-        <f>SUM(G12:G16)</f>
-        <v>2440</v>
-      </c>
-      <c r="H17" s="15"/>
+        <v>7621</v>
+      </c>
+      <c r="F17" s="16"/>
+      <c r="G17" s="18"/>
+      <c r="H17" s="16"/>
     </row>
     <row r="18">
       <c r="A18" s="4" t="s">
-        <v>32</v>
-      </c>
-      <c r="B18" s="20" t="s">
         <v>33</v>
+      </c>
+      <c r="B18" s="21" t="s">
+        <v>34</v>
       </c>
       <c r="C18" s="6">
         <v>1.0</v>
@@ -1132,24 +1047,21 @@
         <v>5499.0</v>
       </c>
       <c r="E18" s="8">
-        <f t="shared" ref="E18:E24" si="5">C18*D18</f>
+        <f t="shared" ref="E18:E24" si="4">C18*D18</f>
         <v>5499</v>
       </c>
-      <c r="F18" s="6">
-        <v>45.0</v>
-      </c>
-      <c r="G18" s="8">
-        <f>C18*F18</f>
-        <v>45</v>
-      </c>
-      <c r="H18" s="10" t="s">
-        <v>34</v>
+      <c r="F18" s="6"/>
+      <c r="G18" s="10">
+        <v>17.0</v>
+      </c>
+      <c r="H18" s="11" t="s">
+        <v>35</v>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="11"/>
-      <c r="B19" s="20" t="s">
-        <v>35</v>
+      <c r="A19" s="12"/>
+      <c r="B19" s="21" t="s">
+        <v>36</v>
       </c>
       <c r="C19" s="6">
         <v>1.0</v>
@@ -1158,45 +1070,44 @@
         <v>6639.0</v>
       </c>
       <c r="E19" s="8">
-        <f t="shared" si="5"/>
+        <f t="shared" si="4"/>
         <v>6639</v>
       </c>
       <c r="F19" s="6"/>
-      <c r="G19" s="8"/>
-      <c r="H19" s="10" t="s">
-        <v>36</v>
+      <c r="G19" s="10">
+        <v>20.0</v>
+      </c>
+      <c r="H19" s="11" t="s">
+        <v>37</v>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="11"/>
-      <c r="B20" s="18" t="s">
-        <v>37</v>
+      <c r="A20" s="12"/>
+      <c r="B20" s="22" t="s">
+        <v>38</v>
       </c>
       <c r="C20" s="9">
         <v>1.0</v>
       </c>
       <c r="D20" s="7">
-        <v>6819.0</v>
+        <v>10999.0</v>
       </c>
       <c r="E20" s="8">
-        <f t="shared" si="5"/>
-        <v>6819</v>
-      </c>
-      <c r="F20" s="6">
-        <v>420.0</v>
-      </c>
-      <c r="G20" s="8">
-        <f t="shared" ref="G20:G24" si="6">C20*F20</f>
-        <v>420</v>
-      </c>
-      <c r="H20" s="10" t="s">
-        <v>38</v>
+        <f t="shared" si="4"/>
+        <v>10999</v>
+      </c>
+      <c r="F20" s="9"/>
+      <c r="G20" s="10">
+        <v>720.0</v>
+      </c>
+      <c r="H20" s="11" t="s">
+        <v>39</v>
       </c>
     </row>
     <row r="21" ht="15.75" customHeight="1">
-      <c r="A21" s="11"/>
-      <c r="B21" s="12" t="s">
-        <v>39</v>
+      <c r="A21" s="12"/>
+      <c r="B21" s="13" t="s">
+        <v>40</v>
       </c>
       <c r="C21" s="6">
         <v>1.0</v>
@@ -1205,24 +1116,19 @@
         <v>500.0</v>
       </c>
       <c r="E21" s="8">
-        <f t="shared" si="5"/>
+        <f t="shared" si="4"/>
         <v>500</v>
       </c>
-      <c r="F21" s="6">
-        <v>25.0</v>
-      </c>
-      <c r="G21" s="8">
-        <f t="shared" si="6"/>
-        <v>25</v>
-      </c>
-      <c r="H21" s="14" t="s">
-        <v>28</v>
+      <c r="F21" s="6"/>
+      <c r="G21" s="8"/>
+      <c r="H21" s="15" t="s">
+        <v>29</v>
       </c>
     </row>
     <row r="22" ht="15.75" customHeight="1">
-      <c r="A22" s="11"/>
-      <c r="B22" s="12" t="s">
-        <v>40</v>
+      <c r="A22" s="12"/>
+      <c r="B22" s="13" t="s">
+        <v>41</v>
       </c>
       <c r="C22" s="6">
         <v>1.0</v>
@@ -1231,50 +1137,40 @@
         <v>1000.0</v>
       </c>
       <c r="E22" s="8">
-        <f t="shared" si="5"/>
+        <f t="shared" si="4"/>
         <v>1000</v>
       </c>
-      <c r="F22" s="6">
-        <v>15.0</v>
-      </c>
-      <c r="G22" s="8">
-        <f t="shared" si="6"/>
-        <v>15</v>
-      </c>
-      <c r="H22" s="14" t="s">
-        <v>28</v>
+      <c r="F22" s="6"/>
+      <c r="G22" s="8"/>
+      <c r="H22" s="15" t="s">
+        <v>29</v>
       </c>
     </row>
     <row r="23" ht="15.75" customHeight="1">
-      <c r="A23" s="11"/>
-      <c r="B23" s="12" t="s">
-        <v>41</v>
+      <c r="A23" s="12"/>
+      <c r="B23" s="13" t="s">
+        <v>42</v>
       </c>
       <c r="C23" s="6">
         <v>1.0</v>
       </c>
-      <c r="D23" s="13">
+      <c r="D23" s="14">
         <v>600.0</v>
       </c>
       <c r="E23" s="8">
-        <f t="shared" si="5"/>
+        <f t="shared" si="4"/>
         <v>600</v>
       </c>
-      <c r="F23" s="6">
-        <v>15.0</v>
-      </c>
-      <c r="G23" s="8">
-        <f t="shared" si="6"/>
-        <v>15</v>
-      </c>
-      <c r="H23" s="21" t="s">
-        <v>28</v>
+      <c r="F23" s="6"/>
+      <c r="G23" s="8"/>
+      <c r="H23" s="23" t="s">
+        <v>29</v>
       </c>
     </row>
     <row r="24" ht="15.75" customHeight="1">
-      <c r="A24" s="11"/>
+      <c r="A24" s="12"/>
       <c r="B24" s="5" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="C24" s="6">
         <v>1.0</v>
@@ -1283,96 +1179,78 @@
         <v>250.0</v>
       </c>
       <c r="E24" s="8">
-        <f t="shared" si="5"/>
+        <f t="shared" si="4"/>
         <v>250</v>
       </c>
-      <c r="F24" s="6">
-        <v>5.0</v>
-      </c>
-      <c r="G24" s="8">
-        <f t="shared" si="6"/>
-        <v>5</v>
-      </c>
-      <c r="H24" s="14" t="s">
-        <v>28</v>
+      <c r="F24" s="6"/>
+      <c r="G24" s="8"/>
+      <c r="H24" s="15" t="s">
+        <v>29</v>
       </c>
     </row>
     <row r="25" ht="15.75" customHeight="1">
-      <c r="A25" s="15"/>
-      <c r="B25" s="16" t="s">
-        <v>43</v>
-      </c>
-      <c r="C25" s="15"/>
-      <c r="D25" s="15"/>
-      <c r="E25" s="17">
+      <c r="A25" s="16"/>
+      <c r="B25" s="17" t="s">
+        <v>44</v>
+      </c>
+      <c r="C25" s="16"/>
+      <c r="D25" s="16"/>
+      <c r="E25" s="18">
         <f>SUM(E18:E24)</f>
-        <v>21307</v>
-      </c>
-      <c r="F25" s="15"/>
-      <c r="G25" s="17">
-        <f>SUM(G18:G24)</f>
-        <v>525</v>
-      </c>
-      <c r="H25" s="15"/>
+        <v>25487</v>
+      </c>
+      <c r="F25" s="16"/>
+      <c r="G25" s="18"/>
+      <c r="H25" s="16"/>
     </row>
     <row r="26" ht="15.75" customHeight="1">
       <c r="A26" s="4" t="s">
-        <v>44</v>
-      </c>
-      <c r="B26" s="12" t="s">
         <v>45</v>
+      </c>
+      <c r="B26" s="13" t="s">
+        <v>46</v>
       </c>
       <c r="C26" s="6">
         <v>1.0</v>
       </c>
-      <c r="D26" s="13">
+      <c r="D26" s="14">
         <v>900.0</v>
       </c>
       <c r="E26" s="8">
-        <f t="shared" ref="E26:E31" si="7">C26*D26</f>
+        <f t="shared" ref="E26:E31" si="5">C26*D26</f>
         <v>900</v>
       </c>
-      <c r="F26" s="6">
-        <v>130.0</v>
-      </c>
-      <c r="G26" s="8">
-        <f t="shared" ref="G26:G31" si="8">C26*F26</f>
-        <v>130</v>
-      </c>
-      <c r="H26" s="14" t="s">
-        <v>28</v>
+      <c r="F26" s="6"/>
+      <c r="G26" s="8"/>
+      <c r="H26" s="15" t="s">
+        <v>29</v>
       </c>
     </row>
     <row r="27" ht="15.75" customHeight="1">
-      <c r="A27" s="11"/>
+      <c r="A27" s="12"/>
       <c r="B27" s="5" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="C27" s="6">
         <v>1.0</v>
       </c>
-      <c r="D27" s="13">
+      <c r="D27" s="14">
         <v>150.0</v>
       </c>
       <c r="E27" s="8">
-        <f t="shared" si="7"/>
+        <f t="shared" si="5"/>
         <v>150</v>
       </c>
-      <c r="F27" s="6">
-        <v>20.0</v>
-      </c>
-      <c r="G27" s="8">
-        <f t="shared" si="8"/>
-        <v>20</v>
-      </c>
-      <c r="H27" s="14" t="s">
-        <v>28</v>
+      <c r="F27" s="6"/>
+      <c r="G27" s="8"/>
+      <c r="H27" s="15" t="s">
+        <v>29</v>
       </c>
     </row>
     <row r="28" ht="15.75" customHeight="1">
-      <c r="A28" s="11"/>
-      <c r="B28" s="12" t="s">
-        <v>47</v>
+      <c r="A28" s="12"/>
+      <c r="B28" s="13" t="s">
+        <v>48</v>
       </c>
       <c r="C28" s="6">
         <v>3.0</v>
@@ -1381,368 +1259,258 @@
         <v>150.0</v>
       </c>
       <c r="E28" s="8">
-        <f t="shared" si="7"/>
+        <f t="shared" si="5"/>
         <v>450</v>
       </c>
-      <c r="F28" s="6">
-        <v>12.0</v>
-      </c>
-      <c r="G28" s="8">
-        <f t="shared" si="8"/>
-        <v>36</v>
-      </c>
-      <c r="H28" s="14" t="s">
-        <v>28</v>
+      <c r="F28" s="6"/>
+      <c r="G28" s="8"/>
+      <c r="H28" s="15" t="s">
+        <v>29</v>
       </c>
     </row>
     <row r="29" ht="15.75" customHeight="1">
-      <c r="A29" s="11"/>
-      <c r="B29" s="12" t="s">
-        <v>48</v>
+      <c r="A29" s="12"/>
+      <c r="B29" s="13" t="s">
+        <v>49</v>
       </c>
       <c r="C29" s="6">
         <v>1.0</v>
       </c>
-      <c r="D29" s="13">
+      <c r="D29" s="14">
         <v>400.0</v>
       </c>
       <c r="E29" s="8">
-        <f t="shared" si="7"/>
+        <f t="shared" si="5"/>
         <v>400</v>
       </c>
-      <c r="F29" s="6">
-        <v>40.0</v>
-      </c>
-      <c r="G29" s="8">
-        <f t="shared" si="8"/>
-        <v>40</v>
-      </c>
-      <c r="H29" s="14" t="s">
-        <v>28</v>
+      <c r="F29" s="6"/>
+      <c r="G29" s="8"/>
+      <c r="H29" s="15" t="s">
+        <v>29</v>
       </c>
     </row>
     <row r="30" ht="15.75" customHeight="1">
-      <c r="A30" s="11"/>
+      <c r="A30" s="12"/>
       <c r="B30" s="5" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="C30" s="6">
         <v>1.0</v>
       </c>
-      <c r="D30" s="13">
+      <c r="D30" s="14">
         <v>150.0</v>
       </c>
       <c r="E30" s="8">
-        <f t="shared" si="7"/>
+        <f t="shared" si="5"/>
         <v>150</v>
       </c>
-      <c r="F30" s="6">
-        <v>10.0</v>
-      </c>
-      <c r="G30" s="8">
-        <f t="shared" si="8"/>
-        <v>10</v>
-      </c>
-      <c r="H30" s="14" t="s">
-        <v>50</v>
+      <c r="F30" s="6"/>
+      <c r="G30" s="8"/>
+      <c r="H30" s="15" t="s">
+        <v>51</v>
       </c>
     </row>
     <row r="31" ht="15.75" customHeight="1">
-      <c r="A31" s="11"/>
+      <c r="A31" s="12"/>
       <c r="B31" s="5" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="C31" s="6">
         <v>1.0</v>
       </c>
-      <c r="D31" s="13">
+      <c r="D31" s="14">
         <v>200.0</v>
       </c>
       <c r="E31" s="8">
-        <f t="shared" si="7"/>
+        <f t="shared" si="5"/>
         <v>200</v>
       </c>
-      <c r="F31" s="6">
-        <v>15.0</v>
-      </c>
-      <c r="G31" s="8">
-        <f t="shared" si="8"/>
-        <v>15</v>
-      </c>
-      <c r="H31" s="14" t="s">
-        <v>50</v>
+      <c r="F31" s="6"/>
+      <c r="G31" s="8"/>
+      <c r="H31" s="15" t="s">
+        <v>51</v>
       </c>
     </row>
     <row r="32" ht="15.75" customHeight="1">
-      <c r="A32" s="15"/>
-      <c r="B32" s="16" t="s">
-        <v>52</v>
-      </c>
-      <c r="C32" s="15"/>
-      <c r="D32" s="15"/>
-      <c r="E32" s="17">
+      <c r="A32" s="16"/>
+      <c r="B32" s="17" t="s">
+        <v>53</v>
+      </c>
+      <c r="C32" s="16"/>
+      <c r="D32" s="16"/>
+      <c r="E32" s="18">
         <f>SUM(E26:E31)</f>
         <v>2250</v>
       </c>
-      <c r="F32" s="15"/>
-      <c r="G32" s="17">
-        <f>SUM(G26:G31)</f>
-        <v>251</v>
-      </c>
-      <c r="H32" s="15"/>
+      <c r="F32" s="16"/>
+      <c r="G32" s="18"/>
+      <c r="H32" s="16"/>
     </row>
     <row r="33" ht="15.75" customHeight="1">
       <c r="A33" s="4" t="s">
-        <v>53</v>
-      </c>
-      <c r="B33" s="12" t="s">
         <v>54</v>
+      </c>
+      <c r="B33" s="13" t="s">
+        <v>55</v>
       </c>
       <c r="C33" s="6">
         <v>1.0</v>
       </c>
-      <c r="D33" s="13">
+      <c r="D33" s="14">
         <v>500.0</v>
       </c>
       <c r="E33" s="8">
-        <f t="shared" ref="E33:E36" si="9">C33*D33</f>
+        <f t="shared" ref="E33:E36" si="6">C33*D33</f>
         <v>500</v>
       </c>
-      <c r="F33" s="6">
-        <v>80.0</v>
-      </c>
-      <c r="G33" s="8">
-        <f t="shared" ref="G33:G36" si="10">C33*F33</f>
-        <v>80</v>
-      </c>
-      <c r="H33" s="14" t="s">
-        <v>50</v>
+      <c r="F33" s="6"/>
+      <c r="G33" s="8"/>
+      <c r="H33" s="15" t="s">
+        <v>51</v>
       </c>
     </row>
     <row r="34" ht="15.75" customHeight="1">
-      <c r="A34" s="11"/>
-      <c r="B34" s="12" t="s">
-        <v>55</v>
+      <c r="A34" s="12"/>
+      <c r="B34" s="13" t="s">
+        <v>56</v>
       </c>
       <c r="C34" s="6">
         <v>1.0</v>
       </c>
-      <c r="D34" s="13">
+      <c r="D34" s="14">
         <v>250.0</v>
       </c>
       <c r="E34" s="8">
-        <f t="shared" si="9"/>
+        <f t="shared" si="6"/>
         <v>250</v>
       </c>
-      <c r="F34" s="6">
-        <v>25.0</v>
-      </c>
-      <c r="G34" s="8">
-        <f t="shared" si="10"/>
-        <v>25</v>
-      </c>
-      <c r="H34" s="14" t="s">
-        <v>50</v>
+      <c r="F34" s="6"/>
+      <c r="G34" s="8"/>
+      <c r="H34" s="15" t="s">
+        <v>51</v>
       </c>
     </row>
     <row r="35" ht="15.75" customHeight="1">
-      <c r="A35" s="11"/>
-      <c r="B35" s="20" t="s">
-        <v>56</v>
+      <c r="A35" s="12"/>
+      <c r="B35" s="21" t="s">
+        <v>57</v>
       </c>
       <c r="C35" s="6">
         <v>1.0</v>
       </c>
-      <c r="D35" s="13">
+      <c r="D35" s="14">
         <v>350.0</v>
       </c>
       <c r="E35" s="8">
-        <f t="shared" si="9"/>
+        <f t="shared" si="6"/>
         <v>350</v>
       </c>
-      <c r="F35" s="6">
-        <v>30.0</v>
-      </c>
-      <c r="G35" s="8">
-        <f t="shared" si="10"/>
-        <v>30</v>
-      </c>
-      <c r="H35" s="14" t="s">
-        <v>50</v>
+      <c r="F35" s="6"/>
+      <c r="G35" s="8"/>
+      <c r="H35" s="15" t="s">
+        <v>51</v>
       </c>
     </row>
     <row r="36" ht="15.75" customHeight="1">
-      <c r="A36" s="11"/>
-      <c r="B36" s="12" t="s">
-        <v>57</v>
+      <c r="A36" s="12"/>
+      <c r="B36" s="13" t="s">
+        <v>58</v>
       </c>
       <c r="C36" s="6">
         <v>1.0</v>
       </c>
-      <c r="D36" s="13">
+      <c r="D36" s="14">
         <v>250.0</v>
       </c>
       <c r="E36" s="8">
-        <f t="shared" si="9"/>
+        <f t="shared" si="6"/>
         <v>250</v>
       </c>
-      <c r="F36" s="6">
-        <v>15.0</v>
-      </c>
-      <c r="G36" s="8">
-        <f t="shared" si="10"/>
-        <v>15</v>
-      </c>
-      <c r="H36" s="14" t="s">
-        <v>58</v>
+      <c r="F36" s="6"/>
+      <c r="G36" s="8"/>
+      <c r="H36" s="15" t="s">
+        <v>59</v>
       </c>
     </row>
     <row r="37" ht="15.75" customHeight="1">
-      <c r="A37" s="15"/>
-      <c r="B37" s="16" t="s">
-        <v>59</v>
-      </c>
-      <c r="C37" s="15"/>
-      <c r="D37" s="15"/>
-      <c r="E37" s="17">
+      <c r="A37" s="16"/>
+      <c r="B37" s="17" t="s">
+        <v>60</v>
+      </c>
+      <c r="C37" s="16"/>
+      <c r="D37" s="16"/>
+      <c r="E37" s="18">
         <f>SUM(E33:E36)</f>
         <v>1350</v>
       </c>
-      <c r="F37" s="15"/>
-      <c r="G37" s="17">
-        <f>SUM(G33:G36)</f>
-        <v>150</v>
-      </c>
-      <c r="H37" s="15"/>
+      <c r="F37" s="16"/>
+      <c r="G37" s="18"/>
+      <c r="H37" s="16"/>
     </row>
     <row r="38" ht="15.75" customHeight="1">
-      <c r="A38" s="22" t="s">
-        <v>60</v>
-      </c>
-      <c r="B38" s="23" t="s">
+      <c r="A38" s="24" t="s">
         <v>61</v>
       </c>
-      <c r="C38" s="23">
-        <v>6.0</v>
-      </c>
-      <c r="D38" s="23" t="s">
+      <c r="B38" s="24" t="s">
         <v>62</v>
       </c>
-      <c r="E38" s="23">
-        <v>900.0</v>
-      </c>
-      <c r="F38" s="23">
-        <v>6000.0</v>
-      </c>
-      <c r="G38" s="23">
-        <v>6000.0</v>
-      </c>
-      <c r="H38" s="23" t="s">
+      <c r="E38" s="25">
+        <v>22430.0</v>
+      </c>
+      <c r="G38" s="24">
+        <v>3826.6935</v>
+      </c>
+      <c r="H38" s="25" t="s">
         <v>63</v>
       </c>
     </row>
     <row r="39" ht="15.75" customHeight="1">
-      <c r="A39" s="24"/>
-      <c r="B39" s="25" t="s">
+      <c r="A39" s="12"/>
+      <c r="B39" s="26" t="s">
         <v>64</v>
       </c>
-      <c r="C39" s="26">
-        <v>1.8</v>
-      </c>
-      <c r="D39" s="26"/>
-      <c r="E39" s="26">
-        <v>5000.0</v>
-      </c>
-      <c r="F39" s="26">
-        <v>1800.0</v>
-      </c>
-      <c r="G39" s="26">
-        <v>1800.0</v>
-      </c>
-      <c r="H39" s="26" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="40" ht="15.75" customHeight="1">
-      <c r="A40" s="24"/>
-      <c r="B40" s="26" t="s">
+      <c r="C39" s="27"/>
+      <c r="D39" s="27"/>
+      <c r="E39" s="27"/>
+      <c r="F39" s="27"/>
+      <c r="G39" s="28">
+        <v>6521.6935</v>
+      </c>
+      <c r="H39" s="12"/>
+    </row>
+    <row r="40" ht="15.75" customHeight="1"/>
+    <row r="41" ht="15.75" customHeight="1">
+      <c r="B41" s="29" t="s">
         <v>65</v>
       </c>
-      <c r="C40" s="26">
-        <v>8.0</v>
-      </c>
-      <c r="D40" s="27"/>
-      <c r="E40" s="26">
-        <v>10000.0</v>
-      </c>
-      <c r="F40" s="26">
-        <v>8000.0</v>
-      </c>
-      <c r="G40" s="26">
-        <v>8000.0</v>
-      </c>
-      <c r="H40" s="26" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="41" ht="15.75" customHeight="1">
-      <c r="A41" s="28"/>
-      <c r="B41" s="29" t="s">
+      <c r="E41" s="29" t="s">
         <v>66</v>
       </c>
-      <c r="C41" s="28"/>
-      <c r="D41" s="28"/>
-      <c r="E41" s="30">
-        <v>68154.0</v>
-      </c>
-      <c r="F41" s="28"/>
-      <c r="G41" s="31"/>
-      <c r="H41" s="28"/>
     </row>
     <row r="42" ht="15.75" customHeight="1">
-      <c r="A42" s="11"/>
-      <c r="B42" s="4"/>
-      <c r="C42" s="11"/>
-      <c r="D42" s="11"/>
-      <c r="E42" s="11"/>
-      <c r="F42" s="11"/>
-      <c r="G42" s="32"/>
-      <c r="H42" s="11"/>
-    </row>
-    <row r="43" ht="15.75" customHeight="1"/>
+      <c r="A42" s="30" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="43" ht="15.75" customHeight="1">
+      <c r="A43" s="2" t="s">
+        <v>68</v>
+      </c>
+    </row>
     <row r="44" ht="15.75" customHeight="1">
-      <c r="B44" s="33" t="s">
-        <v>67</v>
-      </c>
-      <c r="E44" s="33" t="s">
-        <v>68</v>
+      <c r="A44" s="2" t="s">
+        <v>69</v>
       </c>
     </row>
     <row r="45" ht="15.75" customHeight="1">
-      <c r="A45" s="34" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="46" ht="15.75" customHeight="1">
-      <c r="A46" s="2" t="s">
+      <c r="A45" s="31" t="s">
         <v>70</v>
       </c>
     </row>
-    <row r="47" ht="15.75" customHeight="1">
-      <c r="A47" s="35" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="48" ht="15.75" customHeight="1">
-      <c r="A48" s="2" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="49" ht="15.75" customHeight="1">
-      <c r="A49" s="35" t="s">
-        <v>73</v>
-      </c>
-    </row>
+    <row r="46" ht="15.75" customHeight="1"/>
+    <row r="47" ht="15.75" customHeight="1"/>
+    <row r="48" ht="15.75" customHeight="1"/>
+    <row r="49" ht="15.75" customHeight="1"/>
     <row r="50" ht="15.75" customHeight="1"/>
     <row r="51" ht="15.75" customHeight="1"/>
     <row r="52" ht="15.75" customHeight="1"/>
@@ -2688,34 +2456,25 @@
     <row r="992" ht="15.75" customHeight="1"/>
     <row r="993" ht="15.75" customHeight="1"/>
     <row r="994" ht="15.75" customHeight="1"/>
-    <row r="995" ht="15.75" customHeight="1"/>
-    <row r="996" ht="15.75" customHeight="1"/>
-    <row r="997" ht="15.75" customHeight="1"/>
-    <row r="998" ht="15.75" customHeight="1"/>
   </sheetData>
-  <mergeCells count="6">
+  <mergeCells count="5">
     <mergeCell ref="A1:H1"/>
     <mergeCell ref="A2:H2"/>
-    <mergeCell ref="A46:H46"/>
-    <mergeCell ref="A47:H47"/>
-    <mergeCell ref="A48:H48"/>
-    <mergeCell ref="A49:H49"/>
+    <mergeCell ref="A43:H43"/>
+    <mergeCell ref="A44:H44"/>
+    <mergeCell ref="A45:H45"/>
   </mergeCells>
-  <conditionalFormatting sqref="A39:Z40">
-    <cfRule type="notContainsBlanks" dxfId="0" priority="1">
-      <formula>LEN(TRIM(A39))&gt;0</formula>
-    </cfRule>
-  </conditionalFormatting>
   <hyperlinks>
     <hyperlink r:id="rId1" ref="H5"/>
-    <hyperlink r:id="rId2" ref="H13"/>
-    <hyperlink r:id="rId3" ref="H18"/>
-    <hyperlink r:id="rId4" ref="H19"/>
-    <hyperlink r:id="rId5" ref="H20"/>
+    <hyperlink r:id="rId2" ref="H12"/>
+    <hyperlink r:id="rId3" ref="H13"/>
+    <hyperlink r:id="rId4" ref="H18"/>
+    <hyperlink r:id="rId5" ref="H19"/>
+    <hyperlink r:id="rId6" ref="H20"/>
   </hyperlinks>
   <printOptions/>
   <pageMargins bottom="1.0" footer="0.0" header="0.0" left="0.75" right="0.75" top="1.0"/>
   <pageSetup paperSize="9" orientation="portrait"/>
-  <drawing r:id="rId6"/>
+  <drawing r:id="rId7"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
NEW BOM COST OF THE PROJECT REDUCED FROM 725$ TO 525$
</commit_message>
<xml_diff>
--- a/bom/BOM_hado_titan_v3.xlsx
+++ b/bom/BOM_hado_titan_v3.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="85" uniqueCount="71">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="88" uniqueCount="74">
   <si>
     <t>BOM — Haso Titan (India sourcing: Robu.in + Zerodrag) — buffered pricing</t>
   </si>
@@ -43,10 +43,10 @@
     <t>Weapon System</t>
   </si>
   <si>
-    <t>Surpass Hobby Rocket 4092 1250KV brushless motor</t>
-  </si>
-  <si>
-    <t>https://robu.in/product/surpass-hobby-rocket-4092-brushless-rc-car-motor-4pole-%EF%BF%A05-0mm-black-1250-kv/</t>
+    <t>DYS D3548-5 900 KV BLDC Motor</t>
+  </si>
+  <si>
+    <t>https://robu.in/product/dys-d3548-5-900-kv-bldc-motor/</t>
   </si>
   <si>
     <t>HTD 5M pulley, motor side (5mm bore)</t>
@@ -85,10 +85,10 @@
     <t>Drivetrain (x2 sides)</t>
   </si>
   <si>
-    <t>SURPASS HOBBY 3660 ROCKET sensoreless waterproof motor</t>
-  </si>
-  <si>
-    <t>https://www.electropi.in/surpass-hobby-3660-rocket-sensoreless-waterproof-motor-3175-shaft-40-gold-plated-connectors-1750-kv</t>
+    <t>Pro-Range 72.6 N-cm 468 RPM 24V Planetary Gear DC Motor PG36M555-19.2K</t>
+  </si>
+  <si>
+    <t>https://robu.in/product/orange-planetary-gear-dc-motor-24v-468-rpm-72-6-n-cm-pg36m555-19-2k/</t>
   </si>
   <si>
     <t>EasyMech 100mm Modified Heavy Duty Disc Wheel Gray 2 Pc Set</t>
@@ -115,10 +115,16 @@
     <t>Electronics</t>
   </si>
   <si>
-    <t>Zerodrag Boost AM32 55A 4-in-1 ESC (reversible/3D mode)</t>
-  </si>
-  <si>
-    <t>https://zerodrag.in/products/zerodrag-boost-am32-55a-4-in-1-esc-with-12-month-warranty-made-in-india?_pos=1&amp;_sid=d78b98f95&amp;_ss=r</t>
+    <t>SmartElex 30D Smart Motor Driver</t>
+  </si>
+  <si>
+    <t>https://robu.in/product/smartelex-30d-smart-motor-driver-by-raspberry-pi/</t>
+  </si>
+  <si>
+    <t>Readytosky 80A ESC 2-6S Brushless ESC</t>
+  </si>
+  <si>
+    <t>https://robu.in/product/readytosky-80a-esc-2-6s-brushless-esc-speed-controller-for-rc-drone/</t>
   </si>
   <si>
     <t>FlySky FS-i6X (6CH) + FS-iA10B receiver</t>
@@ -127,10 +133,10 @@
     <t>https://robu.in/product/flysky-fs-i6x-2-4ghz-10ch-afhds-2a-rc-transmitter-with-fs-ia10b-2-4ghz-10ch-receiver/</t>
   </si>
   <si>
-    <t>CNHL 5200mAh 22.2V 6S 90C Racing Series Lipo Battery (EC5)</t>
-  </si>
-  <si>
-    <t>https://www.uavstore.in/cnhl-5200mah-22-2v-6s-90c-racing-series-lipo-battery-ec5/</t>
+    <t>GNB 4000mAh 6S1P 22.2V 50C Lipo Battery</t>
+  </si>
+  <si>
+    <t>https://www.uavmarketplace.in/products/gnb-4000mah-6s1p-222v-50c-lipo-battery/895789000000963360</t>
   </si>
   <si>
     <t>Main power switch</t>
@@ -208,10 +214,13 @@
     <t>TOTAL</t>
   </si>
   <si>
+    <t>46087 Rs</t>
+  </si>
+  <si>
     <t>GRAND TOTAL IN USD APPROX</t>
   </si>
   <si>
-    <t>725 USD</t>
+    <t>486 USD</t>
   </si>
   <si>
     <t>Notes</t>
@@ -305,12 +314,6 @@
       <i/>
       <sz val="11.0"/>
       <color rgb="FF93C47D"/>
-      <name val="Rubik"/>
-    </font>
-    <font>
-      <i/>
-      <sz val="11.0"/>
-      <color rgb="FF93C47D"/>
       <name val="&quot;Plus Jakarta Sans&quot;"/>
     </font>
     <font>
@@ -321,8 +324,8 @@
     <font>
       <i/>
       <sz val="11.0"/>
-      <color rgb="FF6AA84F"/>
-      <name val="Inter"/>
+      <color rgb="FF93C47D"/>
+      <name val="Arimo"/>
     </font>
     <font>
       <sz val="8.0"/>
@@ -340,8 +343,15 @@
       <name val="Calibri"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <i/>
+      <sz val="11.0"/>
+      <color rgb="FFEFEFEF"/>
+      <name val="Calibri"/>
+    </font>
   </fonts>
-  <fills count="8">
+  <fills count="7">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -358,12 +368,6 @@
       <patternFill patternType="solid">
         <fgColor rgb="FFD9E1F2"/>
         <bgColor rgb="FFD9E1F2"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFFFF"/>
-        <bgColor rgb="FFFFFFFF"/>
       </patternFill>
     </fill>
     <fill>
@@ -405,7 +409,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="32">
+  <cellXfs count="33">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -422,7 +426,7 @@
       <alignment shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
     <xf borderId="1" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment shrinkToFit="0" vertical="bottom" wrapText="0"/>
+      <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
     <xf borderId="1" fillId="0" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment shrinkToFit="0" vertical="bottom" wrapText="0"/>
@@ -463,37 +467,40 @@
     <xf borderId="1" fillId="3" fontId="4" numFmtId="3" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1" applyNumberFormat="1">
       <alignment shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
-    <xf borderId="0" fillId="4" fontId="12" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
+    <xf borderId="0" fillId="0" fontId="12" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="13" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf borderId="1" fillId="0" fontId="13" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment shrinkToFit="0" vertical="bottom" wrapText="0"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="14" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0" shrinkToFit="0" wrapText="1"/>
+    </xf>
+    <xf borderId="1" fillId="0" fontId="15" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment shrinkToFit="0" vertical="bottom" wrapText="0"/>
+    </xf>
+    <xf borderId="1" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment shrinkToFit="0" vertical="bottom" wrapText="0"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="16" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0"/>
-    </xf>
-    <xf borderId="1" fillId="0" fontId="14" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment shrinkToFit="0" vertical="bottom" wrapText="0"/>
-    </xf>
-    <xf borderId="0" fillId="4" fontId="15" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
-      <alignment readingOrder="0"/>
-    </xf>
-    <xf borderId="1" fillId="0" fontId="16" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="17" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="18" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0"/>
-    </xf>
-    <xf borderId="1" fillId="5" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="1" fillId="4" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
-    <xf borderId="1" fillId="6" fontId="7" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="1" fillId="5" fontId="7" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
-    <xf borderId="1" fillId="7" fontId="4" numFmtId="2" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1" applyNumberFormat="1">
+    <xf borderId="1" fillId="5" fontId="18" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
-    <xf borderId="0" fillId="7" fontId="17" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
+    <xf borderId="1" fillId="6" fontId="4" numFmtId="2" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1" applyNumberFormat="1">
+      <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
+    </xf>
+    <xf borderId="0" fillId="6" fontId="16" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
       <alignment readingOrder="0"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
@@ -774,15 +781,17 @@
         <v>1.0</v>
       </c>
       <c r="D5" s="7">
-        <v>5509.0</v>
+        <v>2709.0</v>
       </c>
       <c r="E5" s="8">
         <f t="shared" ref="E5:E6" si="1">C5*D5</f>
-        <v>5509</v>
-      </c>
-      <c r="F5" s="9"/>
+        <v>2709</v>
+      </c>
+      <c r="F5" s="9">
+        <v>159.0</v>
+      </c>
       <c r="G5" s="10">
-        <v>530.0</v>
+        <v>159.0</v>
       </c>
       <c r="H5" s="11" t="s">
         <v>11</v>
@@ -901,7 +910,7 @@
       <c r="D11" s="16"/>
       <c r="E11" s="18">
         <f>SUM(E5:E10)</f>
-        <v>8087</v>
+        <v>5287</v>
       </c>
       <c r="F11" s="16"/>
       <c r="G11" s="18"/>
@@ -918,15 +927,17 @@
         <v>2.0</v>
       </c>
       <c r="D12" s="7">
-        <v>2100.0</v>
+        <v>1929.0</v>
       </c>
       <c r="E12" s="8">
         <f t="shared" ref="E12:E16" si="3">C12*D12</f>
-        <v>4200</v>
-      </c>
-      <c r="F12" s="9"/>
+        <v>3858</v>
+      </c>
+      <c r="F12" s="9">
+        <v>430.0</v>
+      </c>
       <c r="G12" s="10">
-        <v>976.0</v>
+        <v>860.0</v>
       </c>
       <c r="H12" s="11" t="s">
         <v>25</v>
@@ -934,7 +945,7 @@
     </row>
     <row r="13">
       <c r="A13" s="12"/>
-      <c r="B13" s="20" t="s">
+      <c r="B13" s="19" t="s">
         <v>26</v>
       </c>
       <c r="C13" s="6">
@@ -1027,7 +1038,7 @@
       <c r="D17" s="16"/>
       <c r="E17" s="18">
         <f>SUM(E12:E16)</f>
-        <v>7621</v>
+        <v>7279</v>
       </c>
       <c r="F17" s="16"/>
       <c r="G17" s="18"/>
@@ -1037,22 +1048,24 @@
       <c r="A18" s="4" t="s">
         <v>33</v>
       </c>
-      <c r="B18" s="21" t="s">
+      <c r="B18" s="19" t="s">
         <v>34</v>
       </c>
       <c r="C18" s="6">
         <v>1.0</v>
       </c>
       <c r="D18" s="7">
-        <v>5499.0</v>
+        <v>3269.0</v>
       </c>
       <c r="E18" s="8">
-        <f t="shared" ref="E18:E24" si="4">C18*D18</f>
-        <v>5499</v>
-      </c>
-      <c r="F18" s="6"/>
+        <f>C18*D18</f>
+        <v>3269</v>
+      </c>
+      <c r="F18" s="9">
+        <v>186.0</v>
+      </c>
       <c r="G18" s="10">
-        <v>17.0</v>
+        <v>186.0</v>
       </c>
       <c r="H18" s="11" t="s">
         <v>35</v>
@@ -1060,22 +1073,23 @@
     </row>
     <row r="19">
       <c r="A19" s="12"/>
-      <c r="B19" s="21" t="s">
+      <c r="B19" s="19" t="s">
         <v>36</v>
       </c>
-      <c r="C19" s="6">
+      <c r="C19" s="9">
         <v>1.0</v>
       </c>
       <c r="D19" s="7">
-        <v>6639.0</v>
-      </c>
-      <c r="E19" s="8">
-        <f t="shared" si="4"/>
-        <v>6639</v>
-      </c>
-      <c r="F19" s="6"/>
+        <v>2139.0</v>
+      </c>
+      <c r="E19" s="10">
+        <v>2139.0</v>
+      </c>
+      <c r="F19" s="9">
+        <v>95.0</v>
+      </c>
       <c r="G19" s="10">
-        <v>20.0</v>
+        <v>95.0</v>
       </c>
       <c r="H19" s="11" t="s">
         <v>37</v>
@@ -1083,62 +1097,66 @@
     </row>
     <row r="20">
       <c r="A20" s="12"/>
-      <c r="B20" s="22" t="s">
+      <c r="B20" s="20" t="s">
         <v>38</v>
       </c>
-      <c r="C20" s="9">
+      <c r="C20" s="6">
         <v>1.0</v>
       </c>
       <c r="D20" s="7">
-        <v>10999.0</v>
+        <v>6639.0</v>
       </c>
       <c r="E20" s="8">
-        <f t="shared" si="4"/>
-        <v>10999</v>
-      </c>
-      <c r="F20" s="9"/>
+        <f t="shared" ref="E20:E25" si="4">C20*D20</f>
+        <v>6639</v>
+      </c>
+      <c r="F20" s="6"/>
       <c r="G20" s="10">
-        <v>720.0</v>
+        <v>20.0</v>
       </c>
       <c r="H20" s="11" t="s">
         <v>39</v>
       </c>
     </row>
-    <row r="21" ht="15.75" customHeight="1">
+    <row r="21">
       <c r="A21" s="12"/>
-      <c r="B21" s="13" t="s">
+      <c r="B21" s="21" t="s">
         <v>40</v>
       </c>
-      <c r="C21" s="6">
+      <c r="C21" s="9">
         <v>1.0</v>
       </c>
       <c r="D21" s="7">
-        <v>500.0</v>
+        <v>4569.0</v>
       </c>
       <c r="E21" s="8">
         <f t="shared" si="4"/>
-        <v>500</v>
-      </c>
-      <c r="F21" s="6"/>
-      <c r="G21" s="8"/>
-      <c r="H21" s="15" t="s">
-        <v>29</v>
+        <v>4569</v>
+      </c>
+      <c r="F21" s="9">
+        <v>545.0</v>
+      </c>
+      <c r="G21" s="10">
+        <v>545.0</v>
+      </c>
+      <c r="H21" s="11" t="s">
+        <v>41</v>
       </c>
     </row>
     <row r="22" ht="15.75" customHeight="1">
       <c r="A22" s="12"/>
       <c r="B22" s="13" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C22" s="6">
         <v>1.0</v>
       </c>
       <c r="D22" s="7">
-        <v>1000.0</v>
+        <v>500.0</v>
       </c>
       <c r="E22" s="8">
         <f t="shared" si="4"/>
-        <v>1000</v>
+        <v>500</v>
       </c>
       <c r="F22" s="6"/>
       <c r="G22" s="8"/>
@@ -1149,97 +1167,97 @@
     <row r="23" ht="15.75" customHeight="1">
       <c r="A23" s="12"/>
       <c r="B23" s="13" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="C23" s="6">
         <v>1.0</v>
       </c>
-      <c r="D23" s="14">
-        <v>600.0</v>
+      <c r="D23" s="7">
+        <v>1000.0</v>
       </c>
       <c r="E23" s="8">
         <f t="shared" si="4"/>
-        <v>600</v>
+        <v>1000</v>
       </c>
       <c r="F23" s="6"/>
       <c r="G23" s="8"/>
-      <c r="H23" s="23" t="s">
+      <c r="H23" s="15" t="s">
         <v>29</v>
       </c>
     </row>
     <row r="24" ht="15.75" customHeight="1">
       <c r="A24" s="12"/>
-      <c r="B24" s="5" t="s">
-        <v>43</v>
+      <c r="B24" s="13" t="s">
+        <v>44</v>
       </c>
       <c r="C24" s="6">
         <v>1.0</v>
       </c>
-      <c r="D24" s="7">
-        <v>250.0</v>
+      <c r="D24" s="14">
+        <v>600.0</v>
       </c>
       <c r="E24" s="8">
         <f t="shared" si="4"/>
-        <v>250</v>
+        <v>600</v>
       </c>
       <c r="F24" s="6"/>
       <c r="G24" s="8"/>
-      <c r="H24" s="15" t="s">
+      <c r="H24" s="22" t="s">
         <v>29</v>
       </c>
     </row>
     <row r="25" ht="15.75" customHeight="1">
-      <c r="A25" s="16"/>
-      <c r="B25" s="17" t="s">
-        <v>44</v>
-      </c>
-      <c r="C25" s="16"/>
-      <c r="D25" s="16"/>
-      <c r="E25" s="18">
-        <f>SUM(E18:E24)</f>
-        <v>25487</v>
-      </c>
-      <c r="F25" s="16"/>
-      <c r="G25" s="18"/>
-      <c r="H25" s="16"/>
+      <c r="A25" s="12"/>
+      <c r="B25" s="23" t="s">
+        <v>45</v>
+      </c>
+      <c r="C25" s="6">
+        <v>1.0</v>
+      </c>
+      <c r="D25" s="7">
+        <v>250.0</v>
+      </c>
+      <c r="E25" s="8">
+        <f t="shared" si="4"/>
+        <v>250</v>
+      </c>
+      <c r="F25" s="6"/>
+      <c r="G25" s="8"/>
+      <c r="H25" s="15" t="s">
+        <v>29</v>
+      </c>
     </row>
     <row r="26" ht="15.75" customHeight="1">
-      <c r="A26" s="4" t="s">
-        <v>45</v>
-      </c>
-      <c r="B26" s="13" t="s">
+      <c r="A26" s="16"/>
+      <c r="B26" s="17" t="s">
         <v>46</v>
       </c>
-      <c r="C26" s="6">
-        <v>1.0</v>
-      </c>
-      <c r="D26" s="14">
-        <v>900.0</v>
-      </c>
-      <c r="E26" s="8">
-        <f t="shared" ref="E26:E31" si="5">C26*D26</f>
-        <v>900</v>
-      </c>
-      <c r="F26" s="6"/>
-      <c r="G26" s="8"/>
-      <c r="H26" s="15" t="s">
-        <v>29</v>
-      </c>
+      <c r="C26" s="16"/>
+      <c r="D26" s="16"/>
+      <c r="E26" s="18">
+        <f>SUM(E18:E25)</f>
+        <v>18966</v>
+      </c>
+      <c r="F26" s="16"/>
+      <c r="G26" s="18"/>
+      <c r="H26" s="16"/>
     </row>
     <row r="27" ht="15.75" customHeight="1">
-      <c r="A27" s="12"/>
-      <c r="B27" s="5" t="s">
+      <c r="A27" s="4" t="s">
         <v>47</v>
+      </c>
+      <c r="B27" s="13" t="s">
+        <v>48</v>
       </c>
       <c r="C27" s="6">
         <v>1.0</v>
       </c>
       <c r="D27" s="14">
-        <v>150.0</v>
+        <v>900.0</v>
       </c>
       <c r="E27" s="8">
-        <f t="shared" si="5"/>
-        <v>150</v>
+        <f t="shared" ref="E27:E32" si="5">C27*D27</f>
+        <v>900</v>
       </c>
       <c r="F27" s="6"/>
       <c r="G27" s="8"/>
@@ -1249,18 +1267,18 @@
     </row>
     <row r="28" ht="15.75" customHeight="1">
       <c r="A28" s="12"/>
-      <c r="B28" s="13" t="s">
-        <v>48</v>
+      <c r="B28" s="23" t="s">
+        <v>49</v>
       </c>
       <c r="C28" s="6">
-        <v>3.0</v>
-      </c>
-      <c r="D28" s="7">
+        <v>1.0</v>
+      </c>
+      <c r="D28" s="14">
         <v>150.0</v>
       </c>
       <c r="E28" s="8">
         <f t="shared" si="5"/>
-        <v>450</v>
+        <v>150</v>
       </c>
       <c r="F28" s="6"/>
       <c r="G28" s="8"/>
@@ -1271,17 +1289,17 @@
     <row r="29" ht="15.75" customHeight="1">
       <c r="A29" s="12"/>
       <c r="B29" s="13" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="C29" s="6">
-        <v>1.0</v>
-      </c>
-      <c r="D29" s="14">
-        <v>400.0</v>
+        <v>3.0</v>
+      </c>
+      <c r="D29" s="7">
+        <v>150.0</v>
       </c>
       <c r="E29" s="8">
         <f t="shared" si="5"/>
-        <v>400</v>
+        <v>450</v>
       </c>
       <c r="F29" s="6"/>
       <c r="G29" s="8"/>
@@ -1291,223 +1309,245 @@
     </row>
     <row r="30" ht="15.75" customHeight="1">
       <c r="A30" s="12"/>
-      <c r="B30" s="5" t="s">
-        <v>50</v>
+      <c r="B30" s="13" t="s">
+        <v>51</v>
       </c>
       <c r="C30" s="6">
         <v>1.0</v>
       </c>
       <c r="D30" s="14">
-        <v>150.0</v>
+        <v>400.0</v>
       </c>
       <c r="E30" s="8">
         <f t="shared" si="5"/>
-        <v>150</v>
+        <v>400</v>
       </c>
       <c r="F30" s="6"/>
       <c r="G30" s="8"/>
       <c r="H30" s="15" t="s">
-        <v>51</v>
+        <v>29</v>
       </c>
     </row>
     <row r="31" ht="15.75" customHeight="1">
       <c r="A31" s="12"/>
-      <c r="B31" s="5" t="s">
+      <c r="B31" s="23" t="s">
         <v>52</v>
       </c>
       <c r="C31" s="6">
         <v>1.0</v>
       </c>
       <c r="D31" s="14">
-        <v>200.0</v>
+        <v>150.0</v>
       </c>
       <c r="E31" s="8">
         <f t="shared" si="5"/>
-        <v>200</v>
+        <v>150</v>
       </c>
       <c r="F31" s="6"/>
       <c r="G31" s="8"/>
       <c r="H31" s="15" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
     </row>
     <row r="32" ht="15.75" customHeight="1">
-      <c r="A32" s="16"/>
-      <c r="B32" s="17" t="s">
+      <c r="A32" s="12"/>
+      <c r="B32" s="23" t="s">
+        <v>54</v>
+      </c>
+      <c r="C32" s="6">
+        <v>1.0</v>
+      </c>
+      <c r="D32" s="14">
+        <v>200.0</v>
+      </c>
+      <c r="E32" s="8">
+        <f t="shared" si="5"/>
+        <v>200</v>
+      </c>
+      <c r="F32" s="6"/>
+      <c r="G32" s="8"/>
+      <c r="H32" s="15" t="s">
         <v>53</v>
       </c>
-      <c r="C32" s="16"/>
-      <c r="D32" s="16"/>
-      <c r="E32" s="18">
-        <f>SUM(E26:E31)</f>
+    </row>
+    <row r="33" ht="15.75" customHeight="1">
+      <c r="A33" s="16"/>
+      <c r="B33" s="17" t="s">
+        <v>55</v>
+      </c>
+      <c r="C33" s="16"/>
+      <c r="D33" s="16"/>
+      <c r="E33" s="18">
+        <f>SUM(E27:E32)</f>
         <v>2250</v>
       </c>
-      <c r="F32" s="16"/>
-      <c r="G32" s="18"/>
-      <c r="H32" s="16"/>
-    </row>
-    <row r="33" ht="15.75" customHeight="1">
-      <c r="A33" s="4" t="s">
-        <v>54</v>
-      </c>
-      <c r="B33" s="13" t="s">
-        <v>55</v>
-      </c>
-      <c r="C33" s="6">
-        <v>1.0</v>
-      </c>
-      <c r="D33" s="14">
-        <v>500.0</v>
-      </c>
-      <c r="E33" s="8">
-        <f t="shared" ref="E33:E36" si="6">C33*D33</f>
-        <v>500</v>
-      </c>
-      <c r="F33" s="6"/>
-      <c r="G33" s="8"/>
-      <c r="H33" s="15" t="s">
-        <v>51</v>
-      </c>
+      <c r="F33" s="16"/>
+      <c r="G33" s="18"/>
+      <c r="H33" s="16"/>
     </row>
     <row r="34" ht="15.75" customHeight="1">
-      <c r="A34" s="12"/>
+      <c r="A34" s="4" t="s">
+        <v>56</v>
+      </c>
       <c r="B34" s="13" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="C34" s="6">
         <v>1.0</v>
       </c>
       <c r="D34" s="14">
-        <v>250.0</v>
+        <v>500.0</v>
       </c>
       <c r="E34" s="8">
-        <f t="shared" si="6"/>
-        <v>250</v>
+        <f t="shared" ref="E34:E37" si="6">C34*D34</f>
+        <v>500</v>
       </c>
       <c r="F34" s="6"/>
       <c r="G34" s="8"/>
       <c r="H34" s="15" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
     </row>
     <row r="35" ht="15.75" customHeight="1">
       <c r="A35" s="12"/>
-      <c r="B35" s="21" t="s">
-        <v>57</v>
+      <c r="B35" s="13" t="s">
+        <v>58</v>
       </c>
       <c r="C35" s="6">
         <v>1.0</v>
       </c>
       <c r="D35" s="14">
-        <v>350.0</v>
+        <v>250.0</v>
       </c>
       <c r="E35" s="8">
         <f t="shared" si="6"/>
-        <v>350</v>
+        <v>250</v>
       </c>
       <c r="F35" s="6"/>
       <c r="G35" s="8"/>
       <c r="H35" s="15" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
     </row>
     <row r="36" ht="15.75" customHeight="1">
       <c r="A36" s="12"/>
-      <c r="B36" s="13" t="s">
-        <v>58</v>
+      <c r="B36" s="20" t="s">
+        <v>59</v>
       </c>
       <c r="C36" s="6">
         <v>1.0</v>
       </c>
       <c r="D36" s="14">
-        <v>250.0</v>
+        <v>350.0</v>
       </c>
       <c r="E36" s="8">
         <f t="shared" si="6"/>
-        <v>250</v>
+        <v>350</v>
       </c>
       <c r="F36" s="6"/>
       <c r="G36" s="8"/>
       <c r="H36" s="15" t="s">
-        <v>59</v>
+        <v>53</v>
       </c>
     </row>
     <row r="37" ht="15.75" customHeight="1">
-      <c r="A37" s="16"/>
-      <c r="B37" s="17" t="s">
+      <c r="A37" s="12"/>
+      <c r="B37" s="13" t="s">
         <v>60</v>
       </c>
-      <c r="C37" s="16"/>
-      <c r="D37" s="16"/>
-      <c r="E37" s="18">
-        <f>SUM(E33:E36)</f>
+      <c r="C37" s="6">
+        <v>1.0</v>
+      </c>
+      <c r="D37" s="14">
+        <v>250.0</v>
+      </c>
+      <c r="E37" s="8">
+        <f t="shared" si="6"/>
+        <v>250</v>
+      </c>
+      <c r="F37" s="6"/>
+      <c r="G37" s="8"/>
+      <c r="H37" s="15" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="38" ht="15.75" customHeight="1">
+      <c r="A38" s="16"/>
+      <c r="B38" s="17" t="s">
+        <v>62</v>
+      </c>
+      <c r="C38" s="16"/>
+      <c r="D38" s="16"/>
+      <c r="E38" s="18">
+        <f>SUM(E34:E37)</f>
         <v>1350</v>
       </c>
-      <c r="F37" s="16"/>
-      <c r="G37" s="18"/>
-      <c r="H37" s="16"/>
-    </row>
-    <row r="38" ht="15.75" customHeight="1">
-      <c r="A38" s="24" t="s">
-        <v>61</v>
-      </c>
-      <c r="B38" s="24" t="s">
-        <v>62</v>
-      </c>
-      <c r="E38" s="25">
-        <v>22430.0</v>
-      </c>
-      <c r="G38" s="24">
-        <v>3826.6935</v>
-      </c>
-      <c r="H38" s="25" t="s">
+      <c r="F38" s="16"/>
+      <c r="G38" s="18"/>
+      <c r="H38" s="16"/>
+    </row>
+    <row r="39" ht="15.75" customHeight="1">
+      <c r="A39" s="24" t="s">
         <v>63</v>
       </c>
-    </row>
-    <row r="39" ht="15.75" customHeight="1">
-      <c r="A39" s="12"/>
-      <c r="B39" s="26" t="s">
+      <c r="B39" s="24" t="s">
         <v>64</v>
       </c>
-      <c r="C39" s="27"/>
-      <c r="D39" s="27"/>
-      <c r="E39" s="27"/>
-      <c r="F39" s="27"/>
-      <c r="G39" s="28">
+      <c r="E39" s="25">
+        <v>15000.0</v>
+      </c>
+      <c r="G39" s="24">
+        <v>1676.41</v>
+      </c>
+      <c r="H39" s="25" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="40" ht="15.75" customHeight="1">
+      <c r="A40" s="12"/>
+      <c r="B40" s="26" t="s">
+        <v>66</v>
+      </c>
+      <c r="C40" s="27"/>
+      <c r="D40" s="27"/>
+      <c r="E40" s="28" t="s">
+        <v>67</v>
+      </c>
+      <c r="F40" s="27"/>
+      <c r="G40" s="29">
         <v>6521.6935</v>
       </c>
-      <c r="H39" s="12"/>
-    </row>
-    <row r="40" ht="15.75" customHeight="1"/>
-    <row r="41" ht="15.75" customHeight="1">
-      <c r="B41" s="29" t="s">
-        <v>65</v>
-      </c>
-      <c r="E41" s="29" t="s">
-        <v>66</v>
-      </c>
-    </row>
+      <c r="H40" s="12"/>
+    </row>
+    <row r="41" ht="15.75" customHeight="1"/>
     <row r="42" ht="15.75" customHeight="1">
-      <c r="A42" s="30" t="s">
-        <v>67</v>
+      <c r="B42" s="30" t="s">
+        <v>68</v>
+      </c>
+      <c r="E42" s="30" t="s">
+        <v>69</v>
       </c>
     </row>
     <row r="43" ht="15.75" customHeight="1">
-      <c r="A43" s="2" t="s">
-        <v>68</v>
+      <c r="A43" s="31" t="s">
+        <v>70</v>
       </c>
     </row>
     <row r="44" ht="15.75" customHeight="1">
       <c r="A44" s="2" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
     </row>
     <row r="45" ht="15.75" customHeight="1">
-      <c r="A45" s="31" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="46" ht="15.75" customHeight="1"/>
+      <c r="A45" s="2" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="46" ht="15.75" customHeight="1">
+      <c r="A46" s="32" t="s">
+        <v>73</v>
+      </c>
+    </row>
     <row r="47" ht="15.75" customHeight="1"/>
     <row r="48" ht="15.75" customHeight="1"/>
     <row r="49" ht="15.75" customHeight="1"/>
@@ -2456,13 +2496,14 @@
     <row r="992" ht="15.75" customHeight="1"/>
     <row r="993" ht="15.75" customHeight="1"/>
     <row r="994" ht="15.75" customHeight="1"/>
+    <row r="995" ht="15.75" customHeight="1"/>
   </sheetData>
   <mergeCells count="5">
     <mergeCell ref="A1:H1"/>
     <mergeCell ref="A2:H2"/>
-    <mergeCell ref="A43:H43"/>
     <mergeCell ref="A44:H44"/>
     <mergeCell ref="A45:H45"/>
+    <mergeCell ref="A46:H46"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink r:id="rId1" ref="H5"/>
@@ -2471,10 +2512,11 @@
     <hyperlink r:id="rId4" ref="H18"/>
     <hyperlink r:id="rId5" ref="H19"/>
     <hyperlink r:id="rId6" ref="H20"/>
+    <hyperlink r:id="rId7" ref="H21"/>
   </hyperlinks>
   <printOptions/>
   <pageMargins bottom="1.0" footer="0.0" header="0.0" left="0.75" right="0.75" top="1.0"/>
   <pageSetup paperSize="9" orientation="portrait"/>
-  <drawing r:id="rId7"/>
+  <drawing r:id="rId8"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
BATTERY BETTER DEAL UPDATED BOM
</commit_message>
<xml_diff>
--- a/bom/BOM_hado_titan_v3.xlsx
+++ b/bom/BOM_hado_titan_v3.xlsx
@@ -133,10 +133,10 @@
     <t>https://robu.in/product/flysky-fs-i6x-2-4ghz-10ch-afhds-2a-rc-transmitter-with-fs-ia10b-2-4ghz-10ch-receiver/</t>
   </si>
   <si>
-    <t>GNB 4000mAh 6S1P 22.2V 50C Lipo Battery</t>
-  </si>
-  <si>
-    <t>https://www.uavmarketplace.in/products/gnb-4000mah-6s1p-222v-50c-lipo-battery/895789000000963360</t>
+    <t>GNB 4000mAh 6S1P 22.2V 70C Lipo Battery</t>
+  </si>
+  <si>
+    <t>https://www.uavmarketplace.in/products/gnb-4000mah-6s1p-22-2v-70c-lipo-battery-xt90/895789000000963405</t>
   </si>
   <si>
     <t>Main power switch</t>
@@ -239,7 +239,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <fonts count="19">
+  <fonts count="18">
     <font>
       <sz val="11.0"/>
       <color theme="1"/>
@@ -322,12 +322,6 @@
       <name val="Arial"/>
     </font>
     <font>
-      <i/>
-      <sz val="11.0"/>
-      <color rgb="FF93C47D"/>
-      <name val="Arimo"/>
-    </font>
-    <font>
       <sz val="8.0"/>
       <color rgb="FF93C47D"/>
       <name val="Arial"/>
@@ -351,7 +345,7 @@
       <name val="Calibri"/>
     </font>
   </fonts>
-  <fills count="7">
+  <fills count="8">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -362,6 +356,12 @@
       <patternFill patternType="solid">
         <fgColor rgb="FF1F4E78"/>
         <bgColor rgb="FF1F4E78"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF274E13"/>
+        <bgColor rgb="FF274E13"/>
       </patternFill>
     </fill>
     <fill>
@@ -409,7 +409,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="33">
+  <cellXfs count="35">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -425,7 +425,7 @@
     <xf borderId="1" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
-    <xf borderId="1" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="1" fillId="3" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
     <xf borderId="1" fillId="0" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
@@ -458,49 +458,55 @@
     <xf borderId="1" fillId="0" fontId="10" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
-    <xf borderId="1" fillId="3" fontId="7" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="1" fillId="4" fontId="7" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
-    <xf borderId="1" fillId="3" fontId="11" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="1" fillId="4" fontId="11" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
-    <xf borderId="1" fillId="3" fontId="4" numFmtId="3" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1" applyNumberFormat="1">
+    <xf borderId="1" fillId="4" fontId="4" numFmtId="3" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1" applyNumberFormat="1">
       <alignment shrinkToFit="0" vertical="bottom" wrapText="0"/>
+    </xf>
+    <xf borderId="0" fillId="3" fontId="12" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
+      <alignment readingOrder="0"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="12" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0"/>
     </xf>
+    <xf borderId="1" fillId="3" fontId="13" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment shrinkToFit="0" vertical="bottom" wrapText="0"/>
+    </xf>
+    <xf borderId="0" fillId="3" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
+      <alignment readingOrder="0" shrinkToFit="0" wrapText="1"/>
+    </xf>
+    <xf borderId="1" fillId="0" fontId="14" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment shrinkToFit="0" vertical="bottom" wrapText="0"/>
+    </xf>
+    <xf borderId="1" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment shrinkToFit="0" vertical="bottom" wrapText="0"/>
+    </xf>
     <xf borderId="1" fillId="0" fontId="13" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="14" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" wrapText="1"/>
-    </xf>
-    <xf borderId="1" fillId="0" fontId="15" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment shrinkToFit="0" vertical="bottom" wrapText="0"/>
-    </xf>
-    <xf borderId="1" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment shrinkToFit="0" vertical="bottom" wrapText="0"/>
+    <xf borderId="0" fillId="0" fontId="15" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="16" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="17" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0"/>
-    </xf>
-    <xf borderId="1" fillId="4" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="1" fillId="5" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
-    <xf borderId="1" fillId="5" fontId="7" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="1" fillId="6" fontId="7" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
-    <xf borderId="1" fillId="5" fontId="18" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="1" fillId="6" fontId="17" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
-    <xf borderId="1" fillId="6" fontId="4" numFmtId="2" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1" applyNumberFormat="1">
+    <xf borderId="1" fillId="7" fontId="4" numFmtId="2" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1" applyNumberFormat="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
-    <xf borderId="0" fillId="6" fontId="16" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
+    <xf borderId="0" fillId="7" fontId="15" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
       <alignment readingOrder="0"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
@@ -945,7 +951,7 @@
     </row>
     <row r="13">
       <c r="A13" s="12"/>
-      <c r="B13" s="19" t="s">
+      <c r="B13" s="20" t="s">
         <v>26</v>
       </c>
       <c r="C13" s="6">
@@ -1097,7 +1103,7 @@
     </row>
     <row r="20">
       <c r="A20" s="12"/>
-      <c r="B20" s="20" t="s">
+      <c r="B20" s="21" t="s">
         <v>38</v>
       </c>
       <c r="C20" s="6">
@@ -1120,18 +1126,18 @@
     </row>
     <row r="21">
       <c r="A21" s="12"/>
-      <c r="B21" s="21" t="s">
+      <c r="B21" s="22" t="s">
         <v>40</v>
       </c>
       <c r="C21" s="9">
         <v>1.0</v>
       </c>
       <c r="D21" s="7">
-        <v>4569.0</v>
+        <v>6900.0</v>
       </c>
       <c r="E21" s="8">
         <f t="shared" si="4"/>
-        <v>4569</v>
+        <v>6900</v>
       </c>
       <c r="F21" s="9">
         <v>545.0</v>
@@ -1202,13 +1208,13 @@
       </c>
       <c r="F24" s="6"/>
       <c r="G24" s="8"/>
-      <c r="H24" s="22" t="s">
+      <c r="H24" s="23" t="s">
         <v>29</v>
       </c>
     </row>
     <row r="25" ht="15.75" customHeight="1">
       <c r="A25" s="12"/>
-      <c r="B25" s="23" t="s">
+      <c r="B25" s="24" t="s">
         <v>45</v>
       </c>
       <c r="C25" s="6">
@@ -1236,7 +1242,7 @@
       <c r="D26" s="16"/>
       <c r="E26" s="18">
         <f>SUM(E18:E25)</f>
-        <v>18966</v>
+        <v>21297</v>
       </c>
       <c r="F26" s="16"/>
       <c r="G26" s="18"/>
@@ -1267,7 +1273,7 @@
     </row>
     <row r="28" ht="15.75" customHeight="1">
       <c r="A28" s="12"/>
-      <c r="B28" s="23" t="s">
+      <c r="B28" s="24" t="s">
         <v>49</v>
       </c>
       <c r="C28" s="6">
@@ -1330,7 +1336,7 @@
     </row>
     <row r="31" ht="15.75" customHeight="1">
       <c r="A31" s="12"/>
-      <c r="B31" s="23" t="s">
+      <c r="B31" s="24" t="s">
         <v>52</v>
       </c>
       <c r="C31" s="6">
@@ -1351,7 +1357,7 @@
     </row>
     <row r="32" ht="15.75" customHeight="1">
       <c r="A32" s="12"/>
-      <c r="B32" s="23" t="s">
+      <c r="B32" s="24" t="s">
         <v>54</v>
       </c>
       <c r="C32" s="6">
@@ -1431,7 +1437,7 @@
     </row>
     <row r="36" ht="15.75" customHeight="1">
       <c r="A36" s="12"/>
-      <c r="B36" s="20" t="s">
+      <c r="B36" s="25" t="s">
         <v>59</v>
       </c>
       <c r="C36" s="6">
@@ -1487,49 +1493,47 @@
       <c r="H38" s="16"/>
     </row>
     <row r="39" ht="15.75" customHeight="1">
-      <c r="A39" s="24" t="s">
+      <c r="A39" s="26" t="s">
         <v>63</v>
       </c>
-      <c r="B39" s="24" t="s">
+      <c r="B39" s="26" t="s">
         <v>64</v>
       </c>
-      <c r="E39" s="25">
+      <c r="E39" s="27">
         <v>15000.0</v>
       </c>
-      <c r="G39" s="24">
+      <c r="G39" s="26">
         <v>1676.41</v>
       </c>
-      <c r="H39" s="25" t="s">
+      <c r="H39" s="27" t="s">
         <v>65</v>
       </c>
     </row>
     <row r="40" ht="15.75" customHeight="1">
       <c r="A40" s="12"/>
-      <c r="B40" s="26" t="s">
+      <c r="B40" s="28" t="s">
         <v>66</v>
       </c>
-      <c r="C40" s="27"/>
-      <c r="D40" s="27"/>
-      <c r="E40" s="28" t="s">
+      <c r="C40" s="29"/>
+      <c r="D40" s="29"/>
+      <c r="E40" s="30" t="s">
         <v>67</v>
       </c>
-      <c r="F40" s="27"/>
-      <c r="G40" s="29">
-        <v>6521.6935</v>
-      </c>
+      <c r="F40" s="29"/>
+      <c r="G40" s="31"/>
       <c r="H40" s="12"/>
     </row>
     <row r="41" ht="15.75" customHeight="1"/>
     <row r="42" ht="15.75" customHeight="1">
-      <c r="B42" s="30" t="s">
+      <c r="B42" s="32" t="s">
         <v>68</v>
       </c>
-      <c r="E42" s="30" t="s">
+      <c r="E42" s="32" t="s">
         <v>69</v>
       </c>
     </row>
     <row r="43" ht="15.75" customHeight="1">
-      <c r="A43" s="31" t="s">
+      <c r="A43" s="33" t="s">
         <v>70</v>
       </c>
     </row>
@@ -1544,7 +1548,7 @@
       </c>
     </row>
     <row r="46" ht="15.75" customHeight="1">
-      <c r="A46" s="32" t="s">
+      <c r="A46" s="34" t="s">
         <v>73</v>
       </c>
     </row>

</xml_diff>

<commit_message>
BOM REDUCED FROM $525 TO $501
</commit_message>
<xml_diff>
--- a/bom/BOM_hado_titan_v3.xlsx
+++ b/bom/BOM_hado_titan_v3.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="88" uniqueCount="74">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="80" uniqueCount="76">
   <si>
     <t>BOM — Haso Titan (India sourcing: Robu.in + Zerodrag) — buffered pricing</t>
   </si>
@@ -91,10 +91,10 @@
     <t>https://robu.in/product/orange-planetary-gear-dc-motor-24v-468-rpm-72-6-n-cm-pg36m555-19-2k/</t>
   </si>
   <si>
-    <t>EasyMech 100mm Modified Heavy Duty Disc Wheel Gray 2 Pc Set</t>
-  </si>
-  <si>
-    <t>https://robu.in/product/modified-heavy-dutyhd-disc-wheel-100mm-dia-2pc-grey-color/</t>
+    <t>EasyMech Heavy Duty 100mm Disc Wheel Gray 2 Pc Set</t>
+  </si>
+  <si>
+    <t>https://robu.in/product/heavy-dutyhd-disc-wheel-100mm-dia-2pc-grey-color/</t>
   </si>
   <si>
     <t>Wheel hub coupling</t>
@@ -139,16 +139,10 @@
     <t>https://www.uavmarketplace.in/products/gnb-4000mah-6s1p-22-2v-70c-lipo-battery-xt90/895789000000963405</t>
   </si>
   <si>
-    <t>Main power switch</t>
-  </si>
-  <si>
     <t>Weapon arming switch/link</t>
   </si>
   <si>
-    <t xml:space="preserve">BEC/UBEC 5-6V </t>
-  </si>
-  <si>
-    <t>Low-voltage alarm</t>
+    <t>https://robu.in/product/toggle-switch-knx-219/</t>
   </si>
   <si>
     <t>Electronics subtotal</t>
@@ -157,46 +151,58 @@
     <t>Wiring &amp; Connectors</t>
   </si>
   <si>
-    <t xml:space="preserve">Silicone wire, 12-14AWG (power) </t>
-  </si>
-  <si>
-    <t>Silicone wire, 22-26AWG (signal)</t>
+    <t>12AWG Solid core insulated wire Silicone-Black and Red</t>
+  </si>
+  <si>
+    <t>https://robu.in/product/high-quality-ultra-flexible-12awg-silicone-wire-red/</t>
+  </si>
+  <si>
+    <t>26AWG High Quality Ultra Flexible Silicone Wire - Black and Red</t>
+  </si>
+  <si>
+    <t>https://robu.in/product/high-quality-ultra-flexible-26awg-silicone-wire-1000m-black/</t>
   </si>
   <si>
     <t>XT90 connectors</t>
   </si>
   <si>
-    <t xml:space="preserve">Bullet connectors, largest size (5mm) </t>
+    <t>Bullet connectors 3.5mm</t>
+  </si>
+  <si>
+    <t>https://robu.in/product/amass-35mm-gold-plated-bullet-battery-connector-pair-gc3510-f-and-gc3510-m/</t>
   </si>
   <si>
     <t>Heat shrink tubing assortment</t>
   </si>
   <si>
+    <t>https://robu.in/product/heat-shrink-sleeve-8mm-red-industrial-grade-woer-hst/</t>
+  </si>
+  <si>
+    <t>Cable sleeving / wire loom</t>
+  </si>
+  <si>
+    <t>https://robu.in/product/nylon-2mm-expandable-braided-sleeve-for-wire-protection-10m-length/</t>
+  </si>
+  <si>
+    <t>Wiring &amp; Connectors subtotal</t>
+  </si>
+  <si>
+    <t>Fasteners &amp; Misc</t>
+  </si>
+  <si>
+    <t>Socket head cap screws, M3-M5 assortment</t>
+  </si>
+  <si>
     <t>Amazon.in — amazon.in</t>
   </si>
   <si>
-    <t>Cable sleeving / wire loom</t>
-  </si>
-  <si>
-    <t>Wiring &amp; Connectors subtotal</t>
-  </si>
-  <si>
-    <t>Fasteners &amp; Misc</t>
-  </si>
-  <si>
-    <t>Socket head cap screws, M3-M5 assortment</t>
-  </si>
-  <si>
     <t xml:space="preserve">Nyloc nuts, M3-M5 assortment </t>
   </si>
   <si>
     <t>Threadlocker (Loctite 243)</t>
   </si>
   <si>
-    <t xml:space="preserve">Keyway stock </t>
-  </si>
-  <si>
-    <t>Local hardware — —</t>
+    <t>https://www.amazon.in/Lock-tite-243-Strength-Heavy-Threadlocker/dp/B0F3XV8P29/ref=sr_1_5?nsdOptOutParam=true&amp;sr=8-5</t>
   </si>
   <si>
     <t>Fasteners &amp; Misc subtotal</t>
@@ -214,13 +220,13 @@
     <t>TOTAL</t>
   </si>
   <si>
-    <t>46087 Rs</t>
+    <t>47903 Rs</t>
   </si>
   <si>
     <t>GRAND TOTAL IN USD APPROX</t>
   </si>
   <si>
-    <t>$525</t>
+    <t>$501</t>
   </si>
   <si>
     <t>Notes</t>
@@ -239,7 +245,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <fonts count="18">
+  <fonts count="19">
     <font>
       <sz val="11.0"/>
       <color theme="1"/>
@@ -322,8 +328,14 @@
       <name val="Arial"/>
     </font>
     <font>
-      <sz val="8.0"/>
+      <sz val="11.0"/>
       <color rgb="FF93C47D"/>
+      <name val="&quot;Plus Jakarta Sans&quot;"/>
+    </font>
+    <font>
+      <i/>
+      <sz val="11.0"/>
+      <color rgb="FF6AA84F"/>
       <name val="Arial"/>
     </font>
     <font>
@@ -345,7 +357,7 @@
       <name val="Calibri"/>
     </font>
   </fonts>
-  <fills count="8">
+  <fills count="9">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -368,6 +380,12 @@
       <patternFill patternType="solid">
         <fgColor rgb="FFD9E1F2"/>
         <bgColor rgb="FFD9E1F2"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF0C343D"/>
+        <bgColor rgb="FF0C343D"/>
       </patternFill>
     </fill>
     <fill>
@@ -409,7 +427,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="35">
+  <cellXfs count="36">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -470,43 +488,46 @@
     <xf borderId="0" fillId="3" fontId="12" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
       <alignment readingOrder="0"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="12" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0"/>
-    </xf>
     <xf borderId="1" fillId="3" fontId="13" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
     <xf borderId="0" fillId="3" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" wrapText="1"/>
     </xf>
-    <xf borderId="1" fillId="0" fontId="14" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="1" fillId="3" fontId="9" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
+    </xf>
+    <xf borderId="0" fillId="3" fontId="14" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
+      <alignment readingOrder="0"/>
+    </xf>
+    <xf borderId="1" fillId="3" fontId="15" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
+    </xf>
+    <xf borderId="1" fillId="3" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
-    <xf borderId="1" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="1" fillId="5" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment shrinkToFit="0" vertical="bottom" wrapText="0"/>
-    </xf>
-    <xf borderId="1" fillId="0" fontId="13" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment shrinkToFit="0" vertical="bottom" wrapText="0"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="15" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="16" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0"/>
     </xf>
-    <xf borderId="1" fillId="5" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="0" fillId="0" fontId="17" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0"/>
+    </xf>
+    <xf borderId="1" fillId="6" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
-    <xf borderId="1" fillId="6" fontId="7" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="1" fillId="7" fontId="7" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
-    <xf borderId="1" fillId="6" fontId="17" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="1" fillId="7" fontId="18" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
-    <xf borderId="1" fillId="7" fontId="4" numFmtId="2" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1" applyNumberFormat="1">
+    <xf borderId="1" fillId="8" fontId="4" numFmtId="2" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1" applyNumberFormat="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
-    <xf borderId="0" fillId="7" fontId="15" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
+    <xf borderId="0" fillId="8" fontId="16" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
       <alignment readingOrder="0"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
@@ -951,18 +972,18 @@
     </row>
     <row r="13">
       <c r="A13" s="12"/>
-      <c r="B13" s="20" t="s">
+      <c r="B13" s="19" t="s">
         <v>26</v>
       </c>
       <c r="C13" s="6">
         <v>1.0</v>
       </c>
       <c r="D13" s="7">
-        <v>1265.0</v>
+        <v>573.0</v>
       </c>
       <c r="E13" s="8">
         <f t="shared" si="3"/>
-        <v>1265</v>
+        <v>573</v>
       </c>
       <c r="F13" s="9"/>
       <c r="G13" s="10">
@@ -1044,7 +1065,7 @@
       <c r="D17" s="16"/>
       <c r="E17" s="18">
         <f>SUM(E12:E16)</f>
-        <v>7279</v>
+        <v>6587</v>
       </c>
       <c r="F17" s="16"/>
       <c r="G17" s="18"/>
@@ -1103,7 +1124,7 @@
     </row>
     <row r="20">
       <c r="A20" s="12"/>
-      <c r="B20" s="21" t="s">
+      <c r="B20" s="20" t="s">
         <v>38</v>
       </c>
       <c r="C20" s="6">
@@ -1113,7 +1134,7 @@
         <v>6639.0</v>
       </c>
       <c r="E20" s="8">
-        <f t="shared" ref="E20:E25" si="4">C20*D20</f>
+        <f t="shared" ref="E20:E22" si="4">C20*D20</f>
         <v>6639</v>
       </c>
       <c r="F20" s="6"/>
@@ -1126,7 +1147,7 @@
     </row>
     <row r="21">
       <c r="A21" s="12"/>
-      <c r="B21" s="22" t="s">
+      <c r="B21" s="21" t="s">
         <v>40</v>
       </c>
       <c r="C21" s="9">
@@ -1151,407 +1172,327 @@
     </row>
     <row r="22" ht="15.75" customHeight="1">
       <c r="A22" s="12"/>
-      <c r="B22" s="13" t="s">
+      <c r="B22" s="22" t="s">
         <v>42</v>
       </c>
       <c r="C22" s="6">
         <v>1.0</v>
       </c>
       <c r="D22" s="7">
-        <v>500.0</v>
+        <v>27.0</v>
       </c>
       <c r="E22" s="8">
         <f t="shared" si="4"/>
-        <v>500</v>
+        <v>27</v>
       </c>
       <c r="F22" s="6"/>
       <c r="G22" s="8"/>
-      <c r="H22" s="15" t="s">
-        <v>29</v>
+      <c r="H22" s="11" t="s">
+        <v>43</v>
       </c>
     </row>
     <row r="23" ht="15.75" customHeight="1">
-      <c r="A23" s="12"/>
-      <c r="B23" s="13" t="s">
-        <v>43</v>
-      </c>
-      <c r="C23" s="6">
-        <v>1.0</v>
-      </c>
-      <c r="D23" s="7">
-        <v>1000.0</v>
-      </c>
-      <c r="E23" s="8">
-        <f t="shared" si="4"/>
-        <v>1000</v>
-      </c>
-      <c r="F23" s="6"/>
-      <c r="G23" s="8"/>
-      <c r="H23" s="15" t="s">
-        <v>29</v>
-      </c>
+      <c r="A23" s="16"/>
+      <c r="B23" s="17" t="s">
+        <v>44</v>
+      </c>
+      <c r="C23" s="16"/>
+      <c r="D23" s="16"/>
+      <c r="E23" s="18">
+        <f>SUM(E18:E22)</f>
+        <v>18974</v>
+      </c>
+      <c r="F23" s="16"/>
+      <c r="G23" s="18"/>
+      <c r="H23" s="16"/>
     </row>
     <row r="24" ht="15.75" customHeight="1">
-      <c r="A24" s="12"/>
-      <c r="B24" s="13" t="s">
-        <v>44</v>
-      </c>
-      <c r="C24" s="6">
-        <v>1.0</v>
-      </c>
-      <c r="D24" s="14">
-        <v>600.0</v>
+      <c r="A24" s="4" t="s">
+        <v>45</v>
+      </c>
+      <c r="B24" s="23" t="s">
+        <v>46</v>
+      </c>
+      <c r="C24" s="9">
+        <v>2.0</v>
+      </c>
+      <c r="D24" s="7">
+        <v>90.0</v>
       </c>
       <c r="E24" s="8">
-        <f t="shared" si="4"/>
-        <v>600</v>
+        <f t="shared" ref="E24:E29" si="5">C24*D24</f>
+        <v>180</v>
       </c>
       <c r="F24" s="6"/>
       <c r="G24" s="8"/>
-      <c r="H24" s="23" t="s">
-        <v>29</v>
+      <c r="H24" s="11" t="s">
+        <v>47</v>
       </c>
     </row>
     <row r="25" ht="15.75" customHeight="1">
       <c r="A25" s="12"/>
-      <c r="B25" s="24" t="s">
-        <v>45</v>
-      </c>
-      <c r="C25" s="6">
-        <v>1.0</v>
+      <c r="B25" s="23" t="s">
+        <v>48</v>
+      </c>
+      <c r="C25" s="9">
+        <v>2.0</v>
       </c>
       <c r="D25" s="7">
-        <v>250.0</v>
+        <v>7.0</v>
       </c>
       <c r="E25" s="8">
-        <f t="shared" si="4"/>
-        <v>250</v>
+        <f t="shared" si="5"/>
+        <v>14</v>
       </c>
       <c r="F25" s="6"/>
       <c r="G25" s="8"/>
-      <c r="H25" s="15" t="s">
+      <c r="H25" s="11" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="26" ht="15.75" customHeight="1">
+      <c r="A26" s="12"/>
+      <c r="B26" s="24" t="s">
+        <v>50</v>
+      </c>
+      <c r="C26" s="9">
+        <v>4.0</v>
+      </c>
+      <c r="D26" s="7">
+        <v>90.0</v>
+      </c>
+      <c r="E26" s="8">
+        <f t="shared" si="5"/>
+        <v>360</v>
+      </c>
+      <c r="F26" s="6"/>
+      <c r="G26" s="8"/>
+      <c r="H26" s="15" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="26" ht="15.75" customHeight="1">
-      <c r="A26" s="16"/>
-      <c r="B26" s="17" t="s">
-        <v>46</v>
-      </c>
-      <c r="C26" s="16"/>
-      <c r="D26" s="16"/>
-      <c r="E26" s="18">
-        <f>SUM(E18:E25)</f>
-        <v>21297</v>
-      </c>
-      <c r="F26" s="16"/>
-      <c r="G26" s="18"/>
-      <c r="H26" s="16"/>
-    </row>
     <row r="27" ht="15.75" customHeight="1">
-      <c r="A27" s="4" t="s">
-        <v>47</v>
-      </c>
-      <c r="B27" s="13" t="s">
-        <v>48</v>
-      </c>
-      <c r="C27" s="6">
-        <v>1.0</v>
-      </c>
-      <c r="D27" s="14">
-        <v>900.0</v>
+      <c r="A27" s="12"/>
+      <c r="B27" s="5" t="s">
+        <v>51</v>
+      </c>
+      <c r="C27" s="9">
+        <v>5.0</v>
+      </c>
+      <c r="D27" s="7">
+        <v>26.0</v>
       </c>
       <c r="E27" s="8">
-        <f t="shared" ref="E27:E32" si="5">C27*D27</f>
-        <v>900</v>
+        <f t="shared" si="5"/>
+        <v>130</v>
       </c>
       <c r="F27" s="6"/>
       <c r="G27" s="8"/>
-      <c r="H27" s="15" t="s">
-        <v>29</v>
+      <c r="H27" s="11" t="s">
+        <v>52</v>
       </c>
     </row>
     <row r="28" ht="15.75" customHeight="1">
       <c r="A28" s="12"/>
-      <c r="B28" s="24" t="s">
-        <v>49</v>
+      <c r="B28" s="25" t="s">
+        <v>53</v>
       </c>
       <c r="C28" s="6">
         <v>1.0</v>
       </c>
-      <c r="D28" s="14">
-        <v>150.0</v>
+      <c r="D28" s="7">
+        <v>30.0</v>
       </c>
       <c r="E28" s="8">
         <f t="shared" si="5"/>
-        <v>150</v>
+        <v>30</v>
       </c>
       <c r="F28" s="6"/>
       <c r="G28" s="8"/>
-      <c r="H28" s="15" t="s">
-        <v>29</v>
+      <c r="H28" s="11" t="s">
+        <v>54</v>
       </c>
     </row>
     <row r="29" ht="15.75" customHeight="1">
       <c r="A29" s="12"/>
-      <c r="B29" s="13" t="s">
-        <v>50</v>
+      <c r="B29" s="26" t="s">
+        <v>55</v>
       </c>
       <c r="C29" s="6">
-        <v>3.0</v>
+        <v>1.0</v>
       </c>
       <c r="D29" s="7">
-        <v>150.0</v>
+        <v>104.0</v>
       </c>
       <c r="E29" s="8">
         <f t="shared" si="5"/>
-        <v>450</v>
+        <v>104</v>
       </c>
       <c r="F29" s="6"/>
       <c r="G29" s="8"/>
-      <c r="H29" s="15" t="s">
-        <v>29</v>
+      <c r="H29" s="11" t="s">
+        <v>56</v>
       </c>
     </row>
     <row r="30" ht="15.75" customHeight="1">
-      <c r="A30" s="12"/>
-      <c r="B30" s="13" t="s">
-        <v>51</v>
-      </c>
-      <c r="C30" s="6">
-        <v>1.0</v>
-      </c>
-      <c r="D30" s="14">
-        <v>400.0</v>
-      </c>
-      <c r="E30" s="8">
-        <f t="shared" si="5"/>
-        <v>400</v>
-      </c>
-      <c r="F30" s="6"/>
-      <c r="G30" s="8"/>
-      <c r="H30" s="15" t="s">
-        <v>29</v>
-      </c>
+      <c r="A30" s="16"/>
+      <c r="B30" s="17" t="s">
+        <v>57</v>
+      </c>
+      <c r="C30" s="16"/>
+      <c r="D30" s="16"/>
+      <c r="E30" s="18">
+        <f>SUM(E24:E29)</f>
+        <v>818</v>
+      </c>
+      <c r="F30" s="16"/>
+      <c r="G30" s="18"/>
+      <c r="H30" s="16"/>
     </row>
     <row r="31" ht="15.75" customHeight="1">
-      <c r="A31" s="12"/>
-      <c r="B31" s="24" t="s">
-        <v>52</v>
+      <c r="A31" s="4" t="s">
+        <v>58</v>
+      </c>
+      <c r="B31" s="13" t="s">
+        <v>59</v>
       </c>
       <c r="C31" s="6">
         <v>1.0</v>
       </c>
       <c r="D31" s="14">
-        <v>150.0</v>
+        <v>500.0</v>
       </c>
       <c r="E31" s="8">
-        <f t="shared" si="5"/>
-        <v>150</v>
+        <f t="shared" ref="E31:E33" si="6">C31*D31</f>
+        <v>500</v>
       </c>
       <c r="F31" s="6"/>
       <c r="G31" s="8"/>
       <c r="H31" s="15" t="s">
-        <v>53</v>
+        <v>60</v>
       </c>
     </row>
     <row r="32" ht="15.75" customHeight="1">
       <c r="A32" s="12"/>
-      <c r="B32" s="24" t="s">
-        <v>54</v>
+      <c r="B32" s="13" t="s">
+        <v>61</v>
       </c>
       <c r="C32" s="6">
         <v>1.0</v>
       </c>
       <c r="D32" s="14">
-        <v>200.0</v>
+        <v>250.0</v>
       </c>
       <c r="E32" s="8">
-        <f t="shared" si="5"/>
-        <v>200</v>
+        <f t="shared" si="6"/>
+        <v>250</v>
       </c>
       <c r="F32" s="6"/>
       <c r="G32" s="8"/>
       <c r="H32" s="15" t="s">
-        <v>53</v>
+        <v>60</v>
       </c>
     </row>
     <row r="33" ht="15.75" customHeight="1">
-      <c r="A33" s="16"/>
-      <c r="B33" s="17" t="s">
-        <v>55</v>
-      </c>
-      <c r="C33" s="16"/>
-      <c r="D33" s="16"/>
-      <c r="E33" s="18">
-        <f>SUM(E27:E32)</f>
-        <v>2250</v>
-      </c>
-      <c r="F33" s="16"/>
-      <c r="G33" s="18"/>
-      <c r="H33" s="16"/>
+      <c r="A33" s="12"/>
+      <c r="B33" s="25" t="s">
+        <v>62</v>
+      </c>
+      <c r="C33" s="6">
+        <v>1.0</v>
+      </c>
+      <c r="D33" s="7">
+        <v>430.0</v>
+      </c>
+      <c r="E33" s="8">
+        <f t="shared" si="6"/>
+        <v>430</v>
+      </c>
+      <c r="F33" s="6"/>
+      <c r="G33" s="8"/>
+      <c r="H33" s="11" t="s">
+        <v>63</v>
+      </c>
     </row>
     <row r="34" ht="15.75" customHeight="1">
-      <c r="A34" s="4" t="s">
-        <v>56</v>
-      </c>
-      <c r="B34" s="13" t="s">
-        <v>57</v>
-      </c>
-      <c r="C34" s="6">
-        <v>1.0</v>
-      </c>
-      <c r="D34" s="14">
-        <v>500.0</v>
-      </c>
-      <c r="E34" s="8">
-        <f t="shared" ref="E34:E37" si="6">C34*D34</f>
-        <v>500</v>
-      </c>
-      <c r="F34" s="6"/>
-      <c r="G34" s="8"/>
-      <c r="H34" s="15" t="s">
-        <v>53</v>
-      </c>
+      <c r="A34" s="16"/>
+      <c r="B34" s="17" t="s">
+        <v>64</v>
+      </c>
+      <c r="C34" s="16"/>
+      <c r="D34" s="16"/>
+      <c r="E34" s="18">
+        <f>SUM(E31:E33)</f>
+        <v>1180</v>
+      </c>
+      <c r="F34" s="16"/>
+      <c r="G34" s="18"/>
+      <c r="H34" s="16"/>
     </row>
     <row r="35" ht="15.75" customHeight="1">
-      <c r="A35" s="12"/>
-      <c r="B35" s="13" t="s">
-        <v>58</v>
-      </c>
-      <c r="C35" s="6">
-        <v>1.0</v>
-      </c>
-      <c r="D35" s="14">
-        <v>250.0</v>
-      </c>
-      <c r="E35" s="8">
-        <f t="shared" si="6"/>
-        <v>250</v>
-      </c>
-      <c r="F35" s="6"/>
-      <c r="G35" s="8"/>
-      <c r="H35" s="15" t="s">
-        <v>53</v>
+      <c r="A35" s="27" t="s">
+        <v>65</v>
+      </c>
+      <c r="B35" s="27" t="s">
+        <v>66</v>
+      </c>
+      <c r="E35" s="28">
+        <v>15000.0</v>
+      </c>
+      <c r="G35" s="27">
+        <v>1676.41</v>
+      </c>
+      <c r="H35" s="28" t="s">
+        <v>67</v>
       </c>
     </row>
     <row r="36" ht="15.75" customHeight="1">
       <c r="A36" s="12"/>
-      <c r="B36" s="25" t="s">
-        <v>59</v>
-      </c>
-      <c r="C36" s="6">
-        <v>1.0</v>
-      </c>
-      <c r="D36" s="14">
-        <v>350.0</v>
-      </c>
-      <c r="E36" s="8">
-        <f t="shared" si="6"/>
-        <v>350</v>
-      </c>
-      <c r="F36" s="6"/>
-      <c r="G36" s="8"/>
-      <c r="H36" s="15" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="37" ht="15.75" customHeight="1">
-      <c r="A37" s="12"/>
-      <c r="B37" s="13" t="s">
-        <v>60</v>
-      </c>
-      <c r="C37" s="6">
-        <v>1.0</v>
-      </c>
-      <c r="D37" s="14">
-        <v>250.0</v>
-      </c>
-      <c r="E37" s="8">
-        <f t="shared" si="6"/>
-        <v>250</v>
-      </c>
-      <c r="F37" s="6"/>
-      <c r="G37" s="8"/>
-      <c r="H37" s="15" t="s">
-        <v>61</v>
-      </c>
-    </row>
+      <c r="B36" s="29" t="s">
+        <v>68</v>
+      </c>
+      <c r="C36" s="30"/>
+      <c r="D36" s="30"/>
+      <c r="E36" s="31" t="s">
+        <v>69</v>
+      </c>
+      <c r="F36" s="30"/>
+      <c r="G36" s="32"/>
+      <c r="H36" s="12"/>
+    </row>
+    <row r="37" ht="15.75" customHeight="1"/>
     <row r="38" ht="15.75" customHeight="1">
-      <c r="A38" s="16"/>
-      <c r="B38" s="17" t="s">
-        <v>62</v>
-      </c>
-      <c r="C38" s="16"/>
-      <c r="D38" s="16"/>
-      <c r="E38" s="18">
-        <f>SUM(E34:E37)</f>
-        <v>1350</v>
-      </c>
-      <c r="F38" s="16"/>
-      <c r="G38" s="18"/>
-      <c r="H38" s="16"/>
+      <c r="B38" s="33" t="s">
+        <v>70</v>
+      </c>
+      <c r="E38" s="33" t="s">
+        <v>71</v>
+      </c>
     </row>
     <row r="39" ht="15.75" customHeight="1">
-      <c r="A39" s="26" t="s">
-        <v>63</v>
-      </c>
-      <c r="B39" s="26" t="s">
-        <v>64</v>
-      </c>
-      <c r="E39" s="27">
-        <v>15000.0</v>
-      </c>
-      <c r="G39" s="26">
-        <v>1676.41</v>
-      </c>
-      <c r="H39" s="27" t="s">
-        <v>65</v>
+      <c r="A39" s="34" t="s">
+        <v>72</v>
       </c>
     </row>
     <row r="40" ht="15.75" customHeight="1">
-      <c r="A40" s="12"/>
-      <c r="B40" s="28" t="s">
-        <v>66</v>
-      </c>
-      <c r="C40" s="29"/>
-      <c r="D40" s="29"/>
-      <c r="E40" s="30" t="s">
-        <v>67</v>
-      </c>
-      <c r="F40" s="29"/>
-      <c r="G40" s="31"/>
-      <c r="H40" s="12"/>
-    </row>
-    <row r="41" ht="15.75" customHeight="1"/>
+      <c r="A40" s="2" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="41" ht="15.75" customHeight="1">
+      <c r="A41" s="2" t="s">
+        <v>74</v>
+      </c>
+    </row>
     <row r="42" ht="15.75" customHeight="1">
-      <c r="B42" s="32" t="s">
-        <v>68</v>
-      </c>
-      <c r="E42" s="32" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="43" ht="15.75" customHeight="1">
-      <c r="A43" s="33" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="44" ht="15.75" customHeight="1">
-      <c r="A44" s="2" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="45" ht="15.75" customHeight="1">
-      <c r="A45" s="2" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="46" ht="15.75" customHeight="1">
-      <c r="A46" s="34" t="s">
-        <v>73</v>
-      </c>
-    </row>
+      <c r="A42" s="35" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="43" ht="15.75" customHeight="1"/>
+    <row r="44" ht="15.75" customHeight="1"/>
+    <row r="45" ht="15.75" customHeight="1"/>
+    <row r="46" ht="15.75" customHeight="1"/>
     <row r="47" ht="15.75" customHeight="1"/>
     <row r="48" ht="15.75" customHeight="1"/>
     <row r="49" ht="15.75" customHeight="1"/>
@@ -2497,17 +2438,13 @@
     <row r="989" ht="15.75" customHeight="1"/>
     <row r="990" ht="15.75" customHeight="1"/>
     <row r="991" ht="15.75" customHeight="1"/>
-    <row r="992" ht="15.75" customHeight="1"/>
-    <row r="993" ht="15.75" customHeight="1"/>
-    <row r="994" ht="15.75" customHeight="1"/>
-    <row r="995" ht="15.75" customHeight="1"/>
   </sheetData>
   <mergeCells count="5">
     <mergeCell ref="A1:H1"/>
     <mergeCell ref="A2:H2"/>
-    <mergeCell ref="A44:H44"/>
-    <mergeCell ref="A45:H45"/>
-    <mergeCell ref="A46:H46"/>
+    <mergeCell ref="A40:H40"/>
+    <mergeCell ref="A41:H41"/>
+    <mergeCell ref="A42:H42"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink r:id="rId1" ref="H5"/>
@@ -2517,10 +2454,17 @@
     <hyperlink r:id="rId5" ref="H19"/>
     <hyperlink r:id="rId6" ref="H20"/>
     <hyperlink r:id="rId7" ref="H21"/>
+    <hyperlink r:id="rId8" ref="H22"/>
+    <hyperlink r:id="rId9" ref="H24"/>
+    <hyperlink r:id="rId10" ref="H25"/>
+    <hyperlink r:id="rId11" ref="H27"/>
+    <hyperlink r:id="rId12" ref="H28"/>
+    <hyperlink r:id="rId13" ref="H29"/>
+    <hyperlink r:id="rId14" ref="H33"/>
   </hyperlinks>
   <printOptions/>
   <pageMargins bottom="1.0" footer="0.0" header="0.0" left="0.75" right="0.75" top="1.0"/>
   <pageSetup paperSize="9" orientation="portrait"/>
-  <drawing r:id="rId8"/>
+  <drawing r:id="rId15"/>
 </worksheet>
 </file>
</xml_diff>